<commit_message>
feat: add annuity, annualised capex and toy cost inputs
</commit_message>
<xml_diff>
--- a/data/assumptions_register.xlsx
+++ b/data/assumptions_register.xlsx
@@ -71,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -88,6 +88,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -453,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -515,7 +524,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>re_target_2030</t>
         </is>
@@ -525,15 +534,15 @@
           <t>Renewable share of electricity generation, 2030</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="9" t="n">
         <v>0.35</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -543,12 +552,12 @@
           <t>TAP, 9 Oct 2026: Head of Government reaffirms 35% target</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>https://www.tap.info.tn/fr/Portail-%C3%A0-la-Une-FR-top/20672933-%C3%A9nergie-la</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -560,7 +569,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>flex_cap_mw</t>
         </is>
@@ -570,15 +579,15 @@
           <t>Shiftable load cap (scenario S2-300)</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="9" t="n">
         <v>300</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -588,12 +597,12 @@
           <t>TAP, 9 Oct 2026: action plan targets 300 MW peak-demand reduction</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>https://www.tap.info.tn/fr/Portail-%C3%A0-la-Une-FR-top/20672933-%C3%A9nergie-la</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -605,7 +614,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>flex_cap_hi_mw</t>
         </is>
@@ -615,22 +624,22 @@
           <t>Shiftable load cap, sensitivity (S2-600)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="9" t="n">
         <v>600</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr"/>
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -642,7 +651,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>flex_max_hours</t>
         </is>
@@ -652,22 +661,22 @@
           <t>Maximum shift duration</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr"/>
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -679,7 +688,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>gas_price_factor_lo</t>
         </is>
@@ -689,22 +698,22 @@
           <t>Gas price sensitivity, low</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="9" t="n">
         <v>0.5</v>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>x base</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr"/>
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -716,7 +725,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>gas_price_factor_hi</t>
         </is>
@@ -726,22 +735,22 @@
           <t>Gas price sensitivity, high</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>x base</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr"/>
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -753,7 +762,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>demand_growth</t>
         </is>
@@ -763,15 +772,15 @@
           <t>Electricity demand growth 2022-2030 (CAGR)</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="9" t="n">
         <v>0.037</v>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>1/yr</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -781,12 +790,12 @@
           <t>REGlobal / Renewables Now: Tunisia demand CAGR 3.7% 2022-2030</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>https://reglobal.org/greening-energy-mix-investments-focus-on-increasing-renewables-in-tunisia/</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -798,7 +807,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>peak_ref_2030_mw</t>
         </is>
@@ -808,15 +817,15 @@
           <t>Reference 2030 peak demand</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="9" t="n">
         <v>6000</v>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -826,12 +835,12 @@
           <t>REGlobal / Renewables Now: 6,000 MW peak in 2030</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>https://reglobal.org/greening-energy-mix-investments-focus-on-increasing-renewables-in-tunisia/</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -843,7 +852,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>discount_rate</t>
         </is>
@@ -853,15 +862,15 @@
           <t>Discount rate for annualising investment</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="9" t="n">
         <v>0.07099999999999999</v>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>1/yr</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -871,12 +880,12 @@
           <t>PyPSA-Earth v0.10.0 config.default.yaml, costs.discountrate</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="8" t="inlineStr">
         <is>
           <t>https://github.com/pypsa-meets-earth/pypsa-earth/blob/v0.10.0/config.default.yaml</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -888,7 +897,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>demand_2024_twh</t>
         </is>
@@ -898,20 +907,20 @@
           <t>Electricity demand 2024 (generation + net imports)</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr"/>
+      <c r="H11" s="8" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Phase 3: Ember / ONEM.</t>
@@ -919,7 +928,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>imports_2024_twh</t>
         </is>
@@ -929,20 +938,20 @@
           <t>Net electricity imports 2024</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
+      <c r="G12" s="8" t="inlineStr"/>
+      <c r="H12" s="8" t="inlineStr"/>
       <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Phase 3: Ember / ONEM / STEG.</t>
@@ -950,7 +959,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>gas_price_eur_per_mwh_th</t>
         </is>
@@ -960,23 +969,960 @@
           <t>Natural gas price (economic cost)</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>EUR/MWh_th</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="G13" s="8" t="inlineStr"/>
+      <c r="H13" s="8" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Phase 3: technology-data version used by PyPSA-Earth (spec D8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>toy_ccgt_investment</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>CCGT investment</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>1108.7166</v>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>EUR/kW</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>toy_ccgt_fom</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>CCGT fixed O&amp;M</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>3.3494</v>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>%/year</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>toy_ccgt_vom</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>CCGT variable O&amp;M</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>5.6104</v>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>EUR/MWh</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>toy_ccgt_efficiency</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>CCGT electrical efficiency</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>per unit</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, efficiency); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>toy_ccgt_lifetime</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>CCGT lifetime</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>toy_solar_investment</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Utility PV investment</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>482.4785</v>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>EUR/kW_e</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>toy_solar_fom</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Utility PV fixed O&amp;M</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>2.4757</v>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>%/year</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>toy_solar_lifetime</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Utility PV lifetime</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>toy_onwind_investment</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Onshore wind investment</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>1383.3059</v>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>EUR/kW</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>toy_onwind_fom</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Onshore wind fixed O&amp;M</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>1.2167</v>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>%/year</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>toy_onwind_vom</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Onshore wind variable O&amp;M</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>1.8033</v>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>EUR/MWh</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>toy_onwind_lifetime</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Onshore wind lifetime</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>toy_battery_storage_investment</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Battery energy (storage) investment</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>189.861</v>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>EUR/kWh</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery storage, investment); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>toy_battery_storage_lifetime</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Battery energy (storage) lifetime</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery storage, lifetime); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>toy_battery_inverter_investment</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Battery inverter (power) investment</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>213.9279</v>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>EUR/kW</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, investment); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>toy_battery_inverter_fom</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Battery inverter fixed O&amp;M</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>0.3375</v>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>%/year</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, FOM); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>toy_battery_inverter_efficiency</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Battery inverter efficiency (each direction)</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>per unit</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, efficiency); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>toy_battery_inverter_lifetime</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Battery inverter lifetime</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, lifetime); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx, Note K.</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>toy_gas_fuel</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Natural gas fuel cost</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>28.4158</v>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>EUR/MWh_th</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, fuel); original: World Bank (2025) Commodity Markets, https://www.worldbank.org/en/research/commodity-markets; and ENTSO-E &amp; ENTSOG TYNDP 2024 Scenarios Inputs Commodity Prices, https://2024-data.entsos-tyndp-scenarios.eu/files/scenarios-inputs/Prices.zip, accessed: 2026-02-03.</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>toy_gas_co2_intensity</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Natural gas CO2 intensity</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>0.198</v>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>tCO2/MWh_th</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, CO2 intensity); original: Stoichiometric calculation with 50 GJ/t CH4</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>toy_battery_max_hours</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Toy battery energy-to-power ratio</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>assumption</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr"/>
+      <c r="G34" s="8" t="inlineStr"/>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Toy only: fixed storage duration so the battery is one StorageUnit; the full model sizes energy separately.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: battery round-trip efficiency, gas in test fixture, horizon and register checks
</commit_message>
<xml_diff>
--- a/data/assumptions_register.xlsx
+++ b/data/assumptions_register.xlsx
@@ -1717,7 +1717,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Battery inverter efficiency (each direction)</t>
+          <t>Battery round-trip efficiency (source: 'Round trip efficiency DC')</t>
         </is>
       </c>
       <c r="C30" s="9" t="n">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Toy model input (Phase 1); same cost file as PyPSA-Earth v0.10.0.</t>
+          <t>Toy model input (Phase 1); round trip, so each direction uses its square root (as PyPSA-Earth). Source pinned by the v0.15.0 tag.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: add sourced 2024 inputs and committed projects
</commit_message>
<xml_diff>
--- a/data/assumptions_register.xlsx
+++ b/data/assumptions_register.xlsx
@@ -71,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -95,6 +95,12 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -462,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -524,7 +530,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>re_target_2030</t>
         </is>
@@ -534,15 +540,15 @@
           <t>Renewable share of electricity generation, 2030</t>
         </is>
       </c>
-      <c r="C2" s="9" t="n">
+      <c r="C2" s="12" t="n">
         <v>0.35</v>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -552,12 +558,12 @@
           <t>TAP, 9 Oct 2026: Head of Government reaffirms 35% target</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>https://www.tap.info.tn/fr/Portail-%C3%A0-la-Une-FR-top/20672933-%C3%A9nergie-la</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -569,7 +575,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>flex_cap_mw</t>
         </is>
@@ -579,15 +585,15 @@
           <t>Shiftable load cap (scenario S2-300)</t>
         </is>
       </c>
-      <c r="C3" s="9" t="n">
+      <c r="C3" s="12" t="n">
         <v>300</v>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -597,12 +603,12 @@
           <t>TAP, 9 Oct 2026: action plan targets 300 MW peak-demand reduction</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>https://www.tap.info.tn/fr/Portail-%C3%A0-la-Une-FR-top/20672933-%C3%A9nergie-la</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -614,7 +620,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>flex_cap_hi_mw</t>
         </is>
@@ -624,22 +630,22 @@
           <t>Shiftable load cap, sensitivity (S2-600)</t>
         </is>
       </c>
-      <c r="C4" s="9" t="n">
+      <c r="C4" s="12" t="n">
         <v>600</v>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="8" t="inlineStr"/>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr"/>
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -651,7 +657,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>flex_max_hours</t>
         </is>
@@ -661,22 +667,22 @@
           <t>Maximum shift duration</t>
         </is>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="8" t="inlineStr"/>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="G5" s="11" t="inlineStr"/>
+      <c r="H5" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -688,7 +694,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>gas_price_factor_lo</t>
         </is>
@@ -698,22 +704,22 @@
           <t>Gas price sensitivity, low</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>x base</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="8" t="inlineStr"/>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr"/>
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -725,7 +731,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>gas_price_factor_hi</t>
         </is>
@@ -735,22 +741,22 @@
           <t>Gas price sensitivity, high</t>
         </is>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="12" t="n">
         <v>1.5</v>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>x base</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="8" t="inlineStr"/>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr"/>
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -762,7 +768,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>demand_growth</t>
         </is>
@@ -772,15 +778,15 @@
           <t>Electricity demand growth 2022-2030 (CAGR)</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="12" t="n">
         <v>0.037</v>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>1/yr</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -790,24 +796,24 @@
           <t>REGlobal / Renewables Now: Tunisia demand CAGR 3.7% 2022-2030</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>https://reglobal.org/greening-energy-mix-investments-focus-on-increasing-renewables-in-tunisia/</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Secondary (press) source; replace with STEG master plan if obtained (risk R6).</t>
+          <t>REGlobal page names no source for 3.7% (risk R6). Other sources: STEG demand growth 2025 = 4.1% (steg.com.tn/fr/page/produire); government trend 4-5%/yr (pm.gov.tn/en/node/3133, Aug 2026). Author chose STEG's forecast in the JICA 2022 survey if it confirms (~3.2%/yr reported, unverified; needs the JICA download); otherwise 3.7% stays.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>peak_ref_2030_mw</t>
         </is>
@@ -817,15 +823,15 @@
           <t>Reference 2030 peak demand</t>
         </is>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="12" t="n">
         <v>6000</v>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -835,24 +841,24 @@
           <t>REGlobal / Renewables Now: 6,000 MW peak in 2030</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>https://reglobal.org/greening-energy-mix-investments-focus-on-increasing-renewables-in-tunisia/</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="H9" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Used only as a plausibility check (warning, not a constraint).</t>
+          <t>REGlobal page names no source. Measured peaks: 4,888 MW (14 Aug 2024, ONEM/STEG), 4,837 MW (25 Jul 2025, STEG). Used only as a warning check (spec §5.1).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>discount_rate</t>
         </is>
@@ -862,15 +868,15 @@
           <t>Discount rate for annualising investment</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="12" t="n">
         <v>0.07099999999999999</v>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>1/yr</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -880,12 +886,12 @@
           <t>PyPSA-Earth v0.10.0 config.default.yaml, costs.discountrate</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>https://github.com/pypsa-meets-earth/pypsa-earth/blob/v0.10.0/config.default.yaml</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -897,7 +903,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>demand_2024_twh</t>
         </is>
@@ -907,28 +913,42 @@
           <t>Electricity demand 2024 (generation + net imports)</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="C11" s="12" t="n">
+        <v>22.507</v>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="8" t="inlineStr"/>
-      <c r="H11" s="8" t="inlineStr"/>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025), table 'ELECTRICITE', printed p.18</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Phase 3: Ember / ONEM.</t>
+          <t>Sum of the 2024 column (GWh): STEG 18,617 + IPP solar 34 + self-generation solar 557 + third-party purchases 187 + exchanges -1.1 - exports 107.9 + imports 3,221 = 22,507. Excludes self-consumed thermal self-generation. Cross-check: Ember gives 23.96 TWh (gross generation + net imports), about 6% higher. Author chose ONEM (2026-10-28).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>imports_2024_twh</t>
         </is>
@@ -938,28 +958,42 @@
           <t>Net electricity imports 2024</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="C12" s="12" t="n">
+        <v>3.1131</v>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="8" t="inlineStr"/>
-      <c r="H12" s="8" t="inlineStr"/>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025), table 'ELECTRICITE', printed p.18</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Phase 3: Ember / ONEM / STEG.</t>
+          <t>Net imports = imports 3,221 - exports 107.9 GWh (2024). Mainly Algeria and Libya. Cross-check: Ember net imports 2.59 TWh.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>gas_price_eur_per_mwh_th</t>
         </is>
@@ -969,28 +1003,42 @@
           <t>Natural gas price (economic cost)</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="C13" s="12" t="n">
+        <v>28.4158</v>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>EUR/MWh_th</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="8" t="inlineStr"/>
-      <c r="H13" s="8" t="inlineStr"/>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, fuel); original: World Bank Commodity Markets 2025 and ENTSO-E/ENTSOG TYNDP 2024</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Phase 3: technology-data version used by PyPSA-Earth (spec D8).</t>
+          <t>Economic (import-parity) gas price, as used by PyPSA-Earth v0.10.0; not STEG's subsidised tariff (spec D8).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>toy_ccgt_investment</t>
         </is>
@@ -1000,15 +1048,15 @@
           <t>CCGT investment</t>
         </is>
       </c>
-      <c r="C14" s="9" t="n">
+      <c r="C14" s="12" t="n">
         <v>1108.7166</v>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>EUR/kW</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1018,12 +1066,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr">
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="H14" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1035,7 +1083,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>toy_ccgt_fom</t>
         </is>
@@ -1045,15 +1093,15 @@
           <t>CCGT fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C15" s="9" t="n">
+      <c r="C15" s="12" t="n">
         <v>3.3494</v>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1063,12 +1111,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
+      <c r="G15" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
+      <c r="H15" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1080,7 +1128,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>toy_ccgt_vom</t>
         </is>
@@ -1090,15 +1138,15 @@
           <t>CCGT variable O&amp;M</t>
         </is>
       </c>
-      <c r="C16" s="9" t="n">
+      <c r="C16" s="12" t="n">
         <v>5.6104</v>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>EUR/MWh</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1108,12 +1156,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G16" s="8" t="inlineStr">
+      <c r="G16" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="H16" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1125,7 +1173,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>toy_ccgt_efficiency</t>
         </is>
@@ -1135,15 +1183,15 @@
           <t>CCGT electrical efficiency</t>
         </is>
       </c>
-      <c r="C17" s="9" t="n">
+      <c r="C17" s="12" t="n">
         <v>0.58</v>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>per unit</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1153,12 +1201,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, efficiency); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr">
+      <c r="G17" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H17" s="8" t="inlineStr">
+      <c r="H17" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1170,7 +1218,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>toy_ccgt_lifetime</t>
         </is>
@@ -1180,15 +1228,15 @@
           <t>CCGT lifetime</t>
         </is>
       </c>
-      <c r="C18" s="9" t="n">
+      <c r="C18" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1198,12 +1246,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G18" s="8" t="inlineStr">
+      <c r="G18" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H18" s="8" t="inlineStr">
+      <c r="H18" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1215,7 +1263,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>toy_solar_investment</t>
         </is>
@@ -1225,15 +1273,15 @@
           <t>Utility PV investment</t>
         </is>
       </c>
-      <c r="C19" s="9" t="n">
+      <c r="C19" s="12" t="n">
         <v>482.4785</v>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>EUR/kW_e</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1243,12 +1291,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
+      <c r="G19" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="H19" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1260,7 +1308,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>toy_solar_fom</t>
         </is>
@@ -1270,15 +1318,15 @@
           <t>Utility PV fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C20" s="9" t="n">
+      <c r="C20" s="12" t="n">
         <v>2.4757</v>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1288,12 +1336,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G20" s="8" t="inlineStr">
+      <c r="G20" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="H20" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1305,7 +1353,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>toy_solar_lifetime</t>
         </is>
@@ -1315,15 +1363,15 @@
           <t>Utility PV lifetime</t>
         </is>
       </c>
-      <c r="C21" s="9" t="n">
+      <c r="C21" s="12" t="n">
         <v>40</v>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1333,12 +1381,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G21" s="8" t="inlineStr">
+      <c r="G21" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H21" s="8" t="inlineStr">
+      <c r="H21" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1350,7 +1398,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>toy_onwind_investment</t>
         </is>
@@ -1360,15 +1408,15 @@
           <t>Onshore wind investment</t>
         </is>
       </c>
-      <c r="C22" s="9" t="n">
+      <c r="C22" s="12" t="n">
         <v>1383.3059</v>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>EUR/kW</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1378,12 +1426,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G22" s="8" t="inlineStr">
+      <c r="G22" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr">
+      <c r="H22" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1395,7 +1443,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>toy_onwind_fom</t>
         </is>
@@ -1405,15 +1453,15 @@
           <t>Onshore wind fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C23" s="9" t="n">
+      <c r="C23" s="12" t="n">
         <v>1.2167</v>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E23" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1423,12 +1471,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
+      <c r="G23" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H23" s="8" t="inlineStr">
+      <c r="H23" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1440,7 +1488,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>toy_onwind_vom</t>
         </is>
@@ -1450,15 +1498,15 @@
           <t>Onshore wind variable O&amp;M</t>
         </is>
       </c>
-      <c r="C24" s="9" t="n">
+      <c r="C24" s="12" t="n">
         <v>1.8033</v>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>EUR/MWh</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1468,12 +1516,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G24" s="8" t="inlineStr">
+      <c r="G24" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H24" s="8" t="inlineStr">
+      <c r="H24" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1485,7 +1533,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>toy_onwind_lifetime</t>
         </is>
@@ -1495,15 +1543,15 @@
           <t>Onshore wind lifetime</t>
         </is>
       </c>
-      <c r="C25" s="9" t="n">
+      <c r="C25" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1513,12 +1561,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G25" s="8" t="inlineStr">
+      <c r="G25" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H25" s="8" t="inlineStr">
+      <c r="H25" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1530,7 +1578,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>toy_battery_storage_investment</t>
         </is>
@@ -1540,15 +1588,15 @@
           <t>Battery energy (storage) investment</t>
         </is>
       </c>
-      <c r="C26" s="9" t="n">
+      <c r="C26" s="12" t="n">
         <v>189.861</v>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>EUR/kWh</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1558,12 +1606,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery storage, investment); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G26" s="8" t="inlineStr">
+      <c r="G26" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H26" s="8" t="inlineStr">
+      <c r="H26" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1575,7 +1623,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>toy_battery_storage_lifetime</t>
         </is>
@@ -1585,15 +1633,15 @@
           <t>Battery energy (storage) lifetime</t>
         </is>
       </c>
-      <c r="C27" s="9" t="n">
+      <c r="C27" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="D27" s="8" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1603,12 +1651,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery storage, lifetime); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G27" s="8" t="inlineStr">
+      <c r="G27" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H27" s="8" t="inlineStr">
+      <c r="H27" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1620,7 +1668,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>toy_battery_inverter_investment</t>
         </is>
@@ -1630,15 +1678,15 @@
           <t>Battery inverter (power) investment</t>
         </is>
       </c>
-      <c r="C28" s="9" t="n">
+      <c r="C28" s="12" t="n">
         <v>213.9279</v>
       </c>
-      <c r="D28" s="8" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>EUR/kW</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1648,12 +1696,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, investment); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G28" s="8" t="inlineStr">
+      <c r="G28" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H28" s="8" t="inlineStr">
+      <c r="H28" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1665,7 +1713,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>toy_battery_inverter_fom</t>
         </is>
@@ -1675,15 +1723,15 @@
           <t>Battery inverter fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C29" s="9" t="n">
+      <c r="C29" s="12" t="n">
         <v>0.3375</v>
       </c>
-      <c r="D29" s="8" t="inlineStr">
+      <c r="D29" s="11" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E29" s="8" t="inlineStr">
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1693,12 +1741,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, FOM); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G29" s="8" t="inlineStr">
+      <c r="G29" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H29" s="8" t="inlineStr">
+      <c r="H29" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1710,7 +1758,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>toy_battery_inverter_efficiency</t>
         </is>
@@ -1720,15 +1768,15 @@
           <t>Battery round-trip efficiency (source: 'Round trip efficiency DC')</t>
         </is>
       </c>
-      <c r="C30" s="9" t="n">
+      <c r="C30" s="12" t="n">
         <v>0.96</v>
       </c>
-      <c r="D30" s="8" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>per unit</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1738,12 +1786,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, efficiency); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G30" s="8" t="inlineStr">
+      <c r="G30" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H30" s="8" t="inlineStr">
+      <c r="H30" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1755,7 +1803,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>toy_battery_inverter_lifetime</t>
         </is>
@@ -1765,15 +1813,15 @@
           <t>Battery inverter lifetime</t>
         </is>
       </c>
-      <c r="C31" s="9" t="n">
+      <c r="C31" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="D31" s="8" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E31" s="8" t="inlineStr">
+      <c r="E31" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1783,12 +1831,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, lifetime); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx, Note K.</t>
         </is>
       </c>
-      <c r="G31" s="8" t="inlineStr">
+      <c r="G31" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H31" s="8" t="inlineStr">
+      <c r="H31" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1800,7 +1848,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>toy_gas_fuel</t>
         </is>
@@ -1810,15 +1858,15 @@
           <t>Natural gas fuel cost</t>
         </is>
       </c>
-      <c r="C32" s="9" t="n">
+      <c r="C32" s="12" t="n">
         <v>28.4158</v>
       </c>
-      <c r="D32" s="8" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>EUR/MWh_th</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1828,12 +1876,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, fuel); original: World Bank (2025) Commodity Markets, https://www.worldbank.org/en/research/commodity-markets; and ENTSO-E &amp; ENTSOG TYNDP 2024 Scenarios Inputs Commodity Prices, https://2024-data.entsos-tyndp-scenarios.eu/files/scenarios-inputs/Prices.zip, accessed: 2026-02-03.</t>
         </is>
       </c>
-      <c r="G32" s="8" t="inlineStr">
+      <c r="G32" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H32" s="8" t="inlineStr">
+      <c r="H32" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1845,7 +1893,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>toy_gas_co2_intensity</t>
         </is>
@@ -1855,15 +1903,15 @@
           <t>Natural gas CO2 intensity</t>
         </is>
       </c>
-      <c r="C33" s="9" t="n">
+      <c r="C33" s="12" t="n">
         <v>0.198</v>
       </c>
-      <c r="D33" s="8" t="inlineStr">
+      <c r="D33" s="11" t="inlineStr">
         <is>
           <t>tCO2/MWh_th</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
+      <c r="E33" s="11" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1873,12 +1921,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, CO2 intensity); original: Stoichiometric calculation with 50 GJ/t CH4</t>
         </is>
       </c>
-      <c r="G33" s="8" t="inlineStr">
+      <c r="G33" s="11" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H33" s="8" t="inlineStr">
+      <c r="H33" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1890,7 +1938,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>toy_battery_max_hours</t>
         </is>
@@ -1900,22 +1948,22 @@
           <t>Toy battery energy-to-power ratio</t>
         </is>
       </c>
-      <c r="C34" s="9" t="n">
+      <c r="C34" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="D34" s="8" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr"/>
-      <c r="G34" s="8" t="inlineStr"/>
-      <c r="H34" s="8" t="inlineStr">
+      <c r="G34" s="11" t="inlineStr"/>
+      <c r="H34" s="11" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1923,6 +1971,636 @@
       <c r="I34" s="3" t="inlineStr">
         <is>
           <t>Toy only: fixed storage duration so the battery is one StorageUnit; the full model sizes energy separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>cap_2024_ccgt_mw</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Net installed capacity 2024: combined cycle</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="n">
+        <v>2527</v>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H35" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Read from the chart 'Parc de production électrique net 2023-2024', printed p.17 (no text layer). Check: text on the same page says combined cycles are 42% of the fleet; 2527/6012 = 42.0%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>cap_2024_ocgt_mw</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Net installed capacity 2024: gas turbines (open cycle)</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="n">
+        <v>2457</v>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H36" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Read from the chart 'Parc de production électrique net 2023-2024', printed p.17 (no text layer). Check: text on the same page says combined cycles are 42% of the fleet; 2527/6012 = 42.0%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>cap_2024_steam_mw</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Net installed capacity 2024: steam turbines</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="n">
+        <v>660</v>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H37" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Read from the chart 'Parc de production électrique net 2023-2024', printed p.17 (no text layer). Check: text on the same page says combined cycles are 42% of the fleet; 2527/6012 = 42.0%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>cap_2024_re_mw</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Net installed capacity 2024: renewables (hydro + wind + solar, centralised)</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="n">
+        <v>368</v>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H38" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Read from the chart 'Parc de production électrique net 2023-2024', printed p.17 (no text layer). Check: text on the same page says combined cycles are 42% of the fleet; 2527/6012 = 42.0%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>cap_2024_total_mw</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Net installed capacity 2024: total</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="n">
+        <v>6012</v>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H39" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Read from the chart 'Parc de production électrique net 2023-2024', printed p.17 (no text layer). Check: text on the same page says combined cycles are 42% of the fleet; 2527/6012 = 42.0%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>gen_2024_gas_twh</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Electricity generation 2024: natural gas</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="n">
+        <v>18.156</v>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>TWh</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Table 'PRODUCTION D'ELECTRICITE', printed p.18, row GAZ NATUREL. Excludes thermal self-generators.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>gen_2024_oil_twh</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Electricity generation 2024: fuel oil + gasoil</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="n">
+        <v>0.07190000000000001</v>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>TWh</t>
+        </is>
+      </c>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H41" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Same table, row FUEL + GASOIL (71.9 GWh).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>gen_2024_hydro_twh</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Electricity generation 2024: hydro</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t>TWh</t>
+        </is>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H42" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Same table, row HYDRAULIQUE (16 GWh).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>gen_2024_wind_twh</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Electricity generation 2024: wind</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="n">
+        <v>0.337</v>
+      </c>
+      <c r="D43" s="11" t="inlineStr">
+        <is>
+          <t>TWh</t>
+        </is>
+      </c>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H43" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Same table, row EOLIENNE (337 GWh).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>gen_2024_solar_twh</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Electricity generation 2024: solar PV (STEG + IPP + self-generation)</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="n">
+        <v>0.6278</v>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>TWh</t>
+        </is>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H44" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>Same table: STEG solar 36.8 + 'IPP + autoproducteurs (Solaire)' 591 GWh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>gen_2024_total_twh</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Electricity generation 2024: total</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>19.208</v>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>TWh</t>
+        </is>
+      </c>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Same table, row TOTAL (19,208 GWh).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>gas_share_2024</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Gas share of electricity generation 2024</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="n">
+        <v>0.945</v>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H46" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Pie 'Mix de la production électricité pour l'année 2024', printed p.18 (94.5%, including PV self-generation). Denominator = generation. Ember gives 94.52% of generation; ~85% figures elsewhere divide by demand incl. imports (risk R7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>peak_2024_mw</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Peak electricity demand 2024</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="n">
+        <v>4888</v>
+      </c>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="E47" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Printed p.19: record peak of 4888 MW on 14 Aug 2024.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>steg_specific_consumption_2024</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>STEG fleet specific fuel consumption 2024</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="n">
+        <v>194.8</v>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>toe(GCV)/GWh</t>
+        </is>
+      </c>
+      <c r="E48" s="11" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G48" s="11" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H48" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>Table 'Consommation spécifique des moyens de production', printed p.19. Gross calorific value basis. For calibrating fleet efficiency in Task 10.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: validate the 2024 baseline and calibrate fleet, efficiency and demand shape
</commit_message>
<xml_diff>
--- a/data/assumptions_register.xlsx
+++ b/data/assumptions_register.xlsx
@@ -71,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -95,6 +95,18 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -474,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -536,7 +548,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>re_target_2030</t>
         </is>
@@ -546,15 +558,15 @@
           <t>Renewable share of electricity generation, 2030</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n">
+      <c r="C2" s="18" t="n">
         <v>0.35</v>
       </c>
-      <c r="D2" s="13" t="inlineStr">
+      <c r="D2" s="17" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E2" s="13" t="inlineStr">
+      <c r="E2" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -564,12 +576,12 @@
           <t>TAP, 9 Oct 2026: Head of Government reaffirms 35% target</t>
         </is>
       </c>
-      <c r="G2" s="13" t="inlineStr">
+      <c r="G2" s="17" t="inlineStr">
         <is>
           <t>https://www.tap.info.tn/fr/Portail-%C3%A0-la-Une-FR-top/20672933-%C3%A9nergie-la</t>
         </is>
       </c>
-      <c r="H2" s="13" t="inlineStr">
+      <c r="H2" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -581,7 +593,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>flex_cap_mw</t>
         </is>
@@ -591,15 +603,15 @@
           <t>Shiftable load cap (scenario S2-300)</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n">
+      <c r="C3" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -609,12 +621,12 @@
           <t>TAP, 9 Oct 2026: action plan targets 300 MW peak-demand reduction</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>https://www.tap.info.tn/fr/Portail-%C3%A0-la-Une-FR-top/20672933-%C3%A9nergie-la</t>
         </is>
       </c>
-      <c r="H3" s="13" t="inlineStr">
+      <c r="H3" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -626,7 +638,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>flex_cap_hi_mw</t>
         </is>
@@ -636,22 +648,22 @@
           <t>Shiftable load cap, sensitivity (S2-600)</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
+      <c r="C4" s="18" t="n">
         <v>600</v>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="13" t="inlineStr"/>
-      <c r="H4" s="13" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr"/>
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -663,7 +675,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>flex_max_hours</t>
         </is>
@@ -673,22 +685,22 @@
           <t>Maximum shift duration</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
+      <c r="C5" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="13" t="inlineStr"/>
-      <c r="H5" s="13" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr"/>
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -700,7 +712,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>gas_price_factor_lo</t>
         </is>
@@ -710,22 +722,22 @@
           <t>Gas price sensitivity, low</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="D6" s="17" t="inlineStr">
         <is>
           <t>x base</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="13" t="inlineStr"/>
-      <c r="H6" s="13" t="inlineStr">
+      <c r="G6" s="17" t="inlineStr"/>
+      <c r="H6" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -737,7 +749,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>gas_price_factor_hi</t>
         </is>
@@ -747,22 +759,22 @@
           <t>Gas price sensitivity, high</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>x base</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="13" t="inlineStr"/>
-      <c r="H7" s="13" t="inlineStr">
+      <c r="G7" s="17" t="inlineStr"/>
+      <c r="H7" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -774,7 +786,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>demand_growth</t>
         </is>
@@ -784,15 +796,15 @@
           <t>Electricity demand growth 2022-2030 (CAGR)</t>
         </is>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="18" t="n">
         <v>0.032</v>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="17" t="inlineStr">
         <is>
           <t>1/yr</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -802,12 +814,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.2-17 and p.5-34</t>
         </is>
       </c>
-      <c r="G8" s="13" t="inlineStr">
+      <c r="G8" s="17" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H8" s="13" t="inlineStr">
+      <c r="H8" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -819,7 +831,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>peak_ref_2030_mw</t>
         </is>
@@ -829,15 +841,15 @@
           <t>Reference 2030 peak demand</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" s="18" t="n">
         <v>6000</v>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -847,12 +859,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.2-17 and p.5-35</t>
         </is>
       </c>
-      <c r="G9" s="13" t="inlineStr">
+      <c r="G9" s="17" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H9" s="13" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -864,7 +876,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>discount_rate</t>
         </is>
@@ -874,15 +886,15 @@
           <t>Discount rate for annualising investment</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" s="18" t="n">
         <v>0.07099999999999999</v>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>1/yr</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -892,12 +904,12 @@
           <t>PyPSA-Earth v0.10.0 config.default.yaml, costs.discountrate</t>
         </is>
       </c>
-      <c r="G10" s="13" t="inlineStr">
+      <c r="G10" s="17" t="inlineStr">
         <is>
           <t>https://github.com/pypsa-meets-earth/pypsa-earth/blob/v0.10.0/config.default.yaml</t>
         </is>
       </c>
-      <c r="H10" s="13" t="inlineStr">
+      <c r="H10" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -909,7 +921,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>demand_2024_twh</t>
         </is>
@@ -919,15 +931,15 @@
           <t>Electricity demand 2024 (generation + net imports)</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="18" t="n">
         <v>22.507</v>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -937,12 +949,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025), table 'ELECTRICITE', printed p.18</t>
         </is>
       </c>
-      <c r="G11" s="13" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H11" s="13" t="inlineStr">
+      <c r="H11" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -954,7 +966,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>imports_2024_twh</t>
         </is>
@@ -964,15 +976,15 @@
           <t>Net electricity imports 2024</t>
         </is>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="18" t="n">
         <v>3.1131</v>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -982,12 +994,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025), table 'ELECTRICITE', printed p.18</t>
         </is>
       </c>
-      <c r="G12" s="13" t="inlineStr">
+      <c r="G12" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H12" s="13" t="inlineStr">
+      <c r="H12" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -999,7 +1011,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>gas_price_eur_per_mwh_th</t>
         </is>
@@ -1009,15 +1021,15 @@
           <t>Natural gas price (economic cost)</t>
         </is>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="C13" s="18" t="n">
         <v>28.4158</v>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>EUR/MWh_th</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1027,12 +1039,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, fuel); original: World Bank Commodity Markets 2025 and ENTSO-E/ENTSOG TYNDP 2024</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
+      <c r="G13" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H13" s="13" t="inlineStr">
+      <c r="H13" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -1044,7 +1056,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>toy_ccgt_investment</t>
         </is>
@@ -1054,15 +1066,15 @@
           <t>CCGT investment</t>
         </is>
       </c>
-      <c r="C14" s="14" t="n">
+      <c r="C14" s="18" t="n">
         <v>1108.7166</v>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>EUR/kW</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E14" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1072,12 +1084,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G14" s="13" t="inlineStr">
+      <c r="G14" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H14" s="13" t="inlineStr">
+      <c r="H14" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1089,7 +1101,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>toy_ccgt_fom</t>
         </is>
@@ -1099,15 +1111,15 @@
           <t>CCGT fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="C15" s="18" t="n">
         <v>3.3494</v>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E15" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1117,12 +1129,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G15" s="13" t="inlineStr">
+      <c r="G15" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H15" s="13" t="inlineStr">
+      <c r="H15" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1134,7 +1146,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>toy_ccgt_vom</t>
         </is>
@@ -1144,15 +1156,15 @@
           <t>CCGT variable O&amp;M</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n">
+      <c r="C16" s="18" t="n">
         <v>5.6104</v>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D16" s="17" t="inlineStr">
         <is>
           <t>EUR/MWh</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="E16" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1162,12 +1174,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G16" s="13" t="inlineStr">
+      <c r="G16" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H16" s="13" t="inlineStr">
+      <c r="H16" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1179,7 +1191,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>toy_ccgt_efficiency</t>
         </is>
@@ -1189,15 +1201,15 @@
           <t>CCGT electrical efficiency</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n">
+      <c r="C17" s="18" t="n">
         <v>0.58</v>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>per unit</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E17" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1207,12 +1219,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, efficiency); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G17" s="13" t="inlineStr">
+      <c r="G17" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H17" s="13" t="inlineStr">
+      <c r="H17" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1224,7 +1236,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>toy_ccgt_lifetime</t>
         </is>
@@ -1234,15 +1246,15 @@
           <t>CCGT lifetime</t>
         </is>
       </c>
-      <c r="C18" s="14" t="n">
+      <c r="C18" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D18" s="17" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E18" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1252,12 +1264,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G18" s="13" t="inlineStr">
+      <c r="G18" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H18" s="13" t="inlineStr">
+      <c r="H18" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1269,7 +1281,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>toy_solar_investment</t>
         </is>
@@ -1279,15 +1291,15 @@
           <t>Utility PV investment</t>
         </is>
       </c>
-      <c r="C19" s="14" t="n">
+      <c r="C19" s="18" t="n">
         <v>482.4785</v>
       </c>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>EUR/kW_e</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="E19" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1297,12 +1309,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G19" s="13" t="inlineStr">
+      <c r="G19" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H19" s="13" t="inlineStr">
+      <c r="H19" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1314,7 +1326,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>toy_solar_fom</t>
         </is>
@@ -1324,15 +1336,15 @@
           <t>Utility PV fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C20" s="14" t="n">
+      <c r="C20" s="18" t="n">
         <v>2.4757</v>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1342,12 +1354,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G20" s="13" t="inlineStr">
+      <c r="G20" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H20" s="13" t="inlineStr">
+      <c r="H20" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1359,7 +1371,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>toy_solar_lifetime</t>
         </is>
@@ -1369,15 +1381,15 @@
           <t>Utility PV lifetime</t>
         </is>
       </c>
-      <c r="C21" s="14" t="n">
+      <c r="C21" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr">
+      <c r="E21" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1387,12 +1399,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G21" s="13" t="inlineStr">
+      <c r="G21" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H21" s="13" t="inlineStr">
+      <c r="H21" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1404,7 +1416,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>toy_onwind_investment</t>
         </is>
@@ -1414,15 +1426,15 @@
           <t>Onshore wind investment</t>
         </is>
       </c>
-      <c r="C22" s="14" t="n">
+      <c r="C22" s="18" t="n">
         <v>1383.3059</v>
       </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="D22" s="17" t="inlineStr">
         <is>
           <t>EUR/kW</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="E22" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1432,12 +1444,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G22" s="13" t="inlineStr">
+      <c r="G22" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H22" s="13" t="inlineStr">
+      <c r="H22" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1449,7 +1461,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>toy_onwind_fom</t>
         </is>
@@ -1459,15 +1471,15 @@
           <t>Onshore wind fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C23" s="14" t="n">
+      <c r="C23" s="18" t="n">
         <v>1.2167</v>
       </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="D23" s="17" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E23" s="13" t="inlineStr">
+      <c r="E23" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1477,12 +1489,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G23" s="13" t="inlineStr">
+      <c r="G23" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H23" s="13" t="inlineStr">
+      <c r="H23" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1494,7 +1506,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>toy_onwind_vom</t>
         </is>
@@ -1504,15 +1516,15 @@
           <t>Onshore wind variable O&amp;M</t>
         </is>
       </c>
-      <c r="C24" s="14" t="n">
+      <c r="C24" s="18" t="n">
         <v>1.8033</v>
       </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="D24" s="17" t="inlineStr">
         <is>
           <t>EUR/MWh</t>
         </is>
       </c>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="E24" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1522,12 +1534,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G24" s="13" t="inlineStr">
+      <c r="G24" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H24" s="13" t="inlineStr">
+      <c r="H24" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1539,7 +1551,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>toy_onwind_lifetime</t>
         </is>
@@ -1549,15 +1561,15 @@
           <t>Onshore wind lifetime</t>
         </is>
       </c>
-      <c r="C25" s="14" t="n">
+      <c r="C25" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="D25" s="13" t="inlineStr">
+      <c r="D25" s="17" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E25" s="13" t="inlineStr">
+      <c r="E25" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1567,12 +1579,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G25" s="13" t="inlineStr">
+      <c r="G25" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H25" s="13" t="inlineStr">
+      <c r="H25" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1584,7 +1596,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>toy_battery_storage_investment</t>
         </is>
@@ -1594,15 +1606,15 @@
           <t>Battery energy (storage) investment</t>
         </is>
       </c>
-      <c r="C26" s="14" t="n">
+      <c r="C26" s="18" t="n">
         <v>189.861</v>
       </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="D26" s="17" t="inlineStr">
         <is>
           <t>EUR/kWh</t>
         </is>
       </c>
-      <c r="E26" s="13" t="inlineStr">
+      <c r="E26" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1612,12 +1624,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery storage, investment); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G26" s="13" t="inlineStr">
+      <c r="G26" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H26" s="13" t="inlineStr">
+      <c r="H26" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1629,7 +1641,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>toy_battery_storage_lifetime</t>
         </is>
@@ -1639,15 +1651,15 @@
           <t>Battery energy (storage) lifetime</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n">
+      <c r="C27" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="D27" s="17" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E27" s="13" t="inlineStr">
+      <c r="E27" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1657,12 +1669,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery storage, lifetime); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G27" s="13" t="inlineStr">
+      <c r="G27" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H27" s="13" t="inlineStr">
+      <c r="H27" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1674,7 +1686,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>toy_battery_inverter_investment</t>
         </is>
@@ -1684,15 +1696,15 @@
           <t>Battery inverter (power) investment</t>
         </is>
       </c>
-      <c r="C28" s="14" t="n">
+      <c r="C28" s="18" t="n">
         <v>213.9279</v>
       </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="D28" s="17" t="inlineStr">
         <is>
           <t>EUR/kW</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="E28" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1702,12 +1714,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, investment); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G28" s="13" t="inlineStr">
+      <c r="G28" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H28" s="13" t="inlineStr">
+      <c r="H28" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1719,7 +1731,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>toy_battery_inverter_fom</t>
         </is>
@@ -1729,15 +1741,15 @@
           <t>Battery inverter fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
+      <c r="C29" s="18" t="n">
         <v>0.3375</v>
       </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="D29" s="17" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr">
+      <c r="E29" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1747,12 +1759,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, FOM); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G29" s="13" t="inlineStr">
+      <c r="G29" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H29" s="13" t="inlineStr">
+      <c r="H29" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1764,7 +1776,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>toy_battery_inverter_efficiency</t>
         </is>
@@ -1774,15 +1786,15 @@
           <t>Battery round-trip efficiency (source: 'Round trip efficiency DC')</t>
         </is>
       </c>
-      <c r="C30" s="14" t="n">
+      <c r="C30" s="18" t="n">
         <v>0.96</v>
       </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="D30" s="17" t="inlineStr">
         <is>
           <t>per unit</t>
         </is>
       </c>
-      <c r="E30" s="13" t="inlineStr">
+      <c r="E30" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1792,12 +1804,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, efficiency); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G30" s="13" t="inlineStr">
+      <c r="G30" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H30" s="13" t="inlineStr">
+      <c r="H30" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1809,7 +1821,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>toy_battery_inverter_lifetime</t>
         </is>
@@ -1819,15 +1831,15 @@
           <t>Battery inverter lifetime</t>
         </is>
       </c>
-      <c r="C31" s="14" t="n">
+      <c r="C31" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="D31" s="13" t="inlineStr">
+      <c r="D31" s="17" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E31" s="13" t="inlineStr">
+      <c r="E31" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1837,12 +1849,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, lifetime); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx, Note K.</t>
         </is>
       </c>
-      <c r="G31" s="13" t="inlineStr">
+      <c r="G31" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H31" s="13" t="inlineStr">
+      <c r="H31" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1854,7 +1866,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>toy_gas_fuel</t>
         </is>
@@ -1864,15 +1876,15 @@
           <t>Natural gas fuel cost</t>
         </is>
       </c>
-      <c r="C32" s="14" t="n">
+      <c r="C32" s="18" t="n">
         <v>28.4158</v>
       </c>
-      <c r="D32" s="13" t="inlineStr">
+      <c r="D32" s="17" t="inlineStr">
         <is>
           <t>EUR/MWh_th</t>
         </is>
       </c>
-      <c r="E32" s="13" t="inlineStr">
+      <c r="E32" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1882,12 +1894,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, fuel); original: World Bank (2025) Commodity Markets, https://www.worldbank.org/en/research/commodity-markets; and ENTSO-E &amp; ENTSOG TYNDP 2024 Scenarios Inputs Commodity Prices, https://2024-data.entsos-tyndp-scenarios.eu/files/scenarios-inputs/Prices.zip, accessed: 2026-02-03.</t>
         </is>
       </c>
-      <c r="G32" s="13" t="inlineStr">
+      <c r="G32" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H32" s="13" t="inlineStr">
+      <c r="H32" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1899,7 +1911,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>toy_gas_co2_intensity</t>
         </is>
@@ -1909,15 +1921,15 @@
           <t>Natural gas CO2 intensity</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n">
+      <c r="C33" s="18" t="n">
         <v>0.198</v>
       </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="D33" s="17" t="inlineStr">
         <is>
           <t>tCO2/MWh_th</t>
         </is>
       </c>
-      <c r="E33" s="13" t="inlineStr">
+      <c r="E33" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1927,12 +1939,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, CO2 intensity); original: Stoichiometric calculation with 50 GJ/t CH4</t>
         </is>
       </c>
-      <c r="G33" s="13" t="inlineStr">
+      <c r="G33" s="17" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H33" s="13" t="inlineStr">
+      <c r="H33" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1944,7 +1956,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>toy_battery_max_hours</t>
         </is>
@@ -1954,22 +1966,22 @@
           <t>Toy battery energy-to-power ratio</t>
         </is>
       </c>
-      <c r="C34" s="14" t="n">
+      <c r="C34" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="D34" s="17" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="E34" s="13" t="inlineStr">
+      <c r="E34" s="17" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr"/>
-      <c r="G34" s="13" t="inlineStr"/>
-      <c r="H34" s="13" t="inlineStr">
+      <c r="G34" s="17" t="inlineStr"/>
+      <c r="H34" s="17" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1981,7 +1993,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="A35" s="17" t="inlineStr">
         <is>
           <t>cap_2024_ccgt_mw</t>
         </is>
@@ -1991,15 +2003,15 @@
           <t>Net installed capacity 2024: combined cycle</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
+      <c r="C35" s="18" t="n">
         <v>2527</v>
       </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="D35" s="17" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E35" s="13" t="inlineStr">
+      <c r="E35" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2009,12 +2021,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G35" s="13" t="inlineStr">
+      <c r="G35" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H35" s="13" t="inlineStr">
+      <c r="H35" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2026,7 +2038,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="inlineStr">
+      <c r="A36" s="17" t="inlineStr">
         <is>
           <t>cap_2024_ocgt_mw</t>
         </is>
@@ -2036,15 +2048,15 @@
           <t>Net installed capacity 2024: gas turbines (open cycle)</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
+      <c r="C36" s="18" t="n">
         <v>2457</v>
       </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="D36" s="17" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E36" s="13" t="inlineStr">
+      <c r="E36" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2054,12 +2066,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G36" s="13" t="inlineStr">
+      <c r="G36" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H36" s="13" t="inlineStr">
+      <c r="H36" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2071,7 +2083,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>cap_2024_steam_mw</t>
         </is>
@@ -2081,15 +2093,15 @@
           <t>Net installed capacity 2024: steam turbines</t>
         </is>
       </c>
-      <c r="C37" s="14" t="n">
+      <c r="C37" s="18" t="n">
         <v>660</v>
       </c>
-      <c r="D37" s="13" t="inlineStr">
+      <c r="D37" s="17" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E37" s="13" t="inlineStr">
+      <c r="E37" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2099,12 +2111,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G37" s="13" t="inlineStr">
+      <c r="G37" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H37" s="13" t="inlineStr">
+      <c r="H37" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2116,7 +2128,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>cap_2024_re_mw</t>
         </is>
@@ -2126,15 +2138,15 @@
           <t>Net installed capacity 2024: renewables (hydro + wind + solar, centralised)</t>
         </is>
       </c>
-      <c r="C38" s="14" t="n">
+      <c r="C38" s="18" t="n">
         <v>368</v>
       </c>
-      <c r="D38" s="13" t="inlineStr">
+      <c r="D38" s="17" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E38" s="13" t="inlineStr">
+      <c r="E38" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2144,12 +2156,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G38" s="13" t="inlineStr">
+      <c r="G38" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H38" s="13" t="inlineStr">
+      <c r="H38" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2161,7 +2173,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>cap_2024_total_mw</t>
         </is>
@@ -2171,15 +2183,15 @@
           <t>Net installed capacity 2024: total</t>
         </is>
       </c>
-      <c r="C39" s="14" t="n">
+      <c r="C39" s="18" t="n">
         <v>6012</v>
       </c>
-      <c r="D39" s="13" t="inlineStr">
+      <c r="D39" s="17" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E39" s="13" t="inlineStr">
+      <c r="E39" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2189,12 +2201,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G39" s="13" t="inlineStr">
+      <c r="G39" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H39" s="13" t="inlineStr">
+      <c r="H39" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2206,7 +2218,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="A40" s="17" t="inlineStr">
         <is>
           <t>gen_2024_gas_twh</t>
         </is>
@@ -2216,15 +2228,15 @@
           <t>Electricity generation 2024: natural gas</t>
         </is>
       </c>
-      <c r="C40" s="14" t="n">
+      <c r="C40" s="18" t="n">
         <v>18.156</v>
       </c>
-      <c r="D40" s="13" t="inlineStr">
+      <c r="D40" s="17" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E40" s="13" t="inlineStr">
+      <c r="E40" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2234,12 +2246,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G40" s="13" t="inlineStr">
+      <c r="G40" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H40" s="13" t="inlineStr">
+      <c r="H40" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2251,7 +2263,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="13" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>gen_2024_oil_twh</t>
         </is>
@@ -2261,15 +2273,15 @@
           <t>Electricity generation 2024: fuel oil + gasoil</t>
         </is>
       </c>
-      <c r="C41" s="14" t="n">
+      <c r="C41" s="18" t="n">
         <v>0.07190000000000001</v>
       </c>
-      <c r="D41" s="13" t="inlineStr">
+      <c r="D41" s="17" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E41" s="13" t="inlineStr">
+      <c r="E41" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2279,12 +2291,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G41" s="13" t="inlineStr">
+      <c r="G41" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H41" s="13" t="inlineStr">
+      <c r="H41" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2296,7 +2308,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="A42" s="17" t="inlineStr">
         <is>
           <t>gen_2024_hydro_twh</t>
         </is>
@@ -2306,15 +2318,15 @@
           <t>Electricity generation 2024: hydro</t>
         </is>
       </c>
-      <c r="C42" s="14" t="n">
+      <c r="C42" s="18" t="n">
         <v>0.016</v>
       </c>
-      <c r="D42" s="13" t="inlineStr">
+      <c r="D42" s="17" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E42" s="13" t="inlineStr">
+      <c r="E42" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2324,12 +2336,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G42" s="13" t="inlineStr">
+      <c r="G42" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H42" s="13" t="inlineStr">
+      <c r="H42" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2341,7 +2353,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="13" t="inlineStr">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>gen_2024_wind_twh</t>
         </is>
@@ -2351,15 +2363,15 @@
           <t>Electricity generation 2024: wind</t>
         </is>
       </c>
-      <c r="C43" s="14" t="n">
+      <c r="C43" s="18" t="n">
         <v>0.337</v>
       </c>
-      <c r="D43" s="13" t="inlineStr">
+      <c r="D43" s="17" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E43" s="13" t="inlineStr">
+      <c r="E43" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2369,12 +2381,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G43" s="13" t="inlineStr">
+      <c r="G43" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H43" s="13" t="inlineStr">
+      <c r="H43" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2386,7 +2398,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="13" t="inlineStr">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>gen_2024_solar_twh</t>
         </is>
@@ -2396,15 +2408,15 @@
           <t>Electricity generation 2024: solar PV (STEG + IPP + self-generation)</t>
         </is>
       </c>
-      <c r="C44" s="14" t="n">
+      <c r="C44" s="18" t="n">
         <v>0.6278</v>
       </c>
-      <c r="D44" s="13" t="inlineStr">
+      <c r="D44" s="17" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E44" s="13" t="inlineStr">
+      <c r="E44" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2414,12 +2426,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G44" s="13" t="inlineStr">
+      <c r="G44" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H44" s="13" t="inlineStr">
+      <c r="H44" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2431,7 +2443,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="13" t="inlineStr">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>gen_2024_total_twh</t>
         </is>
@@ -2441,15 +2453,15 @@
           <t>Electricity generation 2024: total</t>
         </is>
       </c>
-      <c r="C45" s="14" t="n">
+      <c r="C45" s="18" t="n">
         <v>19.208</v>
       </c>
-      <c r="D45" s="13" t="inlineStr">
+      <c r="D45" s="17" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E45" s="13" t="inlineStr">
+      <c r="E45" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2459,12 +2471,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G45" s="13" t="inlineStr">
+      <c r="G45" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H45" s="13" t="inlineStr">
+      <c r="H45" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2476,7 +2488,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="13" t="inlineStr">
+      <c r="A46" s="17" t="inlineStr">
         <is>
           <t>gas_share_2024</t>
         </is>
@@ -2486,15 +2498,15 @@
           <t>Gas share of electricity generation 2024</t>
         </is>
       </c>
-      <c r="C46" s="14" t="n">
+      <c r="C46" s="18" t="n">
         <v>0.945</v>
       </c>
-      <c r="D46" s="13" t="inlineStr">
+      <c r="D46" s="17" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E46" s="13" t="inlineStr">
+      <c r="E46" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2504,12 +2516,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G46" s="13" t="inlineStr">
+      <c r="G46" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H46" s="13" t="inlineStr">
+      <c r="H46" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2521,7 +2533,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="13" t="inlineStr">
+      <c r="A47" s="17" t="inlineStr">
         <is>
           <t>peak_2024_mw</t>
         </is>
@@ -2531,15 +2543,15 @@
           <t>Peak electricity demand 2024</t>
         </is>
       </c>
-      <c r="C47" s="14" t="n">
+      <c r="C47" s="18" t="n">
         <v>4888</v>
       </c>
-      <c r="D47" s="13" t="inlineStr">
+      <c r="D47" s="17" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E47" s="13" t="inlineStr">
+      <c r="E47" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2549,12 +2561,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G47" s="13" t="inlineStr">
+      <c r="G47" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H47" s="13" t="inlineStr">
+      <c r="H47" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2566,7 +2578,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="13" t="inlineStr">
+      <c r="A48" s="17" t="inlineStr">
         <is>
           <t>steg_specific_consumption_2024</t>
         </is>
@@ -2576,15 +2588,15 @@
           <t>STEG fleet specific fuel consumption 2024</t>
         </is>
       </c>
-      <c r="C48" s="14" t="n">
+      <c r="C48" s="18" t="n">
         <v>194.8</v>
       </c>
-      <c r="D48" s="13" t="inlineStr">
+      <c r="D48" s="17" t="inlineStr">
         <is>
           <t>toe(GCV)/GWh</t>
         </is>
       </c>
-      <c r="E48" s="13" t="inlineStr">
+      <c r="E48" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2594,12 +2606,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G48" s="13" t="inlineStr">
+      <c r="G48" s="17" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H48" s="13" t="inlineStr">
+      <c r="H48" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2611,7 +2623,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="13" t="inlineStr">
+      <c r="A49" s="17" t="inlineStr">
         <is>
           <t>steg_demand_2030_gwh</t>
         </is>
@@ -2621,15 +2633,15 @@
           <t>STEG forecast of 2030 electricity demand</t>
         </is>
       </c>
-      <c r="C49" s="14" t="n">
+      <c r="C49" s="18" t="n">
         <v>28362</v>
       </c>
-      <c r="D49" s="13" t="inlineStr">
+      <c r="D49" s="17" t="inlineStr">
         <is>
           <t>GWh</t>
         </is>
       </c>
-      <c r="E49" s="13" t="inlineStr">
+      <c r="E49" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2639,12 +2651,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.2-17</t>
         </is>
       </c>
-      <c r="G49" s="13" t="inlineStr">
+      <c r="G49" s="17" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H49" s="13" t="inlineStr">
+      <c r="H49" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2656,7 +2668,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="13" t="inlineStr">
+      <c r="A50" s="17" t="inlineStr">
         <is>
           <t>load_factor_2030</t>
         </is>
@@ -2666,15 +2678,15 @@
           <t>STEG 2030 forecast: annual load factor</t>
         </is>
       </c>
-      <c r="C50" s="14" t="n">
+      <c r="C50" s="18" t="n">
         <v>0.54</v>
       </c>
-      <c r="D50" s="13" t="inlineStr">
+      <c r="D50" s="17" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E50" s="13" t="inlineStr">
+      <c r="E50" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2684,12 +2696,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.5-34</t>
         </is>
       </c>
-      <c r="G50" s="13" t="inlineStr">
+      <c r="G50" s="17" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H50" s="13" t="inlineStr">
+      <c r="H50" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2701,7 +2713,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="13" t="inlineStr">
+      <c r="A51" s="17" t="inlineStr">
         <is>
           <t>min_to_peak_2030</t>
         </is>
@@ -2711,15 +2723,15 @@
           <t>STEG 2030 forecast: minimum-to-peak load ratio</t>
         </is>
       </c>
-      <c r="C51" s="14" t="n">
+      <c r="C51" s="18" t="n">
         <v>0.34</v>
       </c>
-      <c r="D51" s="13" t="inlineStr">
+      <c r="D51" s="17" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E51" s="13" t="inlineStr">
+      <c r="E51" s="17" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2729,12 +2741,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.5-35</t>
         </is>
       </c>
-      <c r="G51" s="13" t="inlineStr">
+      <c r="G51" s="17" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H51" s="13" t="inlineStr">
+      <c r="H51" s="17" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2742,6 +2754,276 @@
       <c r="I51" s="3" t="inlineStr">
         <is>
           <t>2030 minimum 2,064 MW (around 7:00 in February) / maximum 6,000 MW = 34% (stated). Shape check (risk R5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>ccgt_efficiency</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>CCGT electrical efficiency (new build)</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>per unit</t>
+        </is>
+      </c>
+      <c r="E52" s="17" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, efficiency); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G52" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H52" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>Same cost file as PyPSA-Earth v0.10.0. Efficiencies are on net calorific value (LHV).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>ccgt_vom</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>CCGT variable O&amp;M</t>
+        </is>
+      </c>
+      <c r="C53" s="18" t="n">
+        <v>5.6104</v>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>EUR/MWh</t>
+        </is>
+      </c>
+      <c r="E53" s="17" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G53" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H53" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Same cost file as PyPSA-Earth v0.10.0. Efficiencies are on net calorific value (LHV).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>ocgt_efficiency</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>OCGT electrical efficiency (new build)</t>
+        </is>
+      </c>
+      <c r="C54" s="18" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>per unit</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (OCGT, efficiency); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G54" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H54" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>Same cost file as PyPSA-Earth v0.10.0. Efficiencies are on net calorific value (LHV).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="inlineStr">
+        <is>
+          <t>ocgt_vom</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>OCGT variable O&amp;M</t>
+        </is>
+      </c>
+      <c r="C55" s="18" t="n">
+        <v>6.0111</v>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
+        <is>
+          <t>EUR/MWh</t>
+        </is>
+      </c>
+      <c r="E55" s="17" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (OCGT, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G55" s="17" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H55" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Same cost file as PyPSA-Earth v0.10.0. Efficiencies are on net calorific value (LHV).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>gas_ncv_per_gcv</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Natural gas: net / gross calorific value</t>
+        </is>
+      </c>
+      <c r="C56" s="18" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="E56" s="17" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024, conversion table (PDF p.22)</t>
+        </is>
+      </c>
+      <c r="G56" s="17" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H56" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>'1PCI = 0,9 PCS'. Converts STEG's specific consumption (gross, PCS) to the net basis of technology-data efficiencies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>existing_gas_efficiency_factor</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Efficiency factor for existing gas units (calibrated)</t>
+        </is>
+      </c>
+      <c r="C57" s="18" t="n">
+        <v>0.8633999999999999</v>
+      </c>
+      <c r="D57" s="17" t="inlineStr">
+        <is>
+          <t>x tech-data</t>
+        </is>
+      </c>
+      <c r="E57" s="17" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Calibrated (Task 10) so the dispatch-only 2024 run matches STEG's measured fuel use: ONEM Memento 2024, specific consumption 194.8 toe(PCS)/GWh, PCI = 0.9 PCS</t>
+        </is>
+      </c>
+      <c r="G57" s="17" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H57" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Computed by scripts/validate_baseline.py: target fleet efficiency 0.490 (net) / model 0.568 at factor 1. Existing CCGT 0.58 x 0.8634 = 0.501; existing OCGT + steam 0.41 x 0.8634 = 0.354. New builds keep tech-data values.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: address Phase 3 review (OCGT new-build option, fuel cross-check, consistent capacities, Phase 4 plan)
</commit_message>
<xml_diff>
--- a/data/assumptions_register.xlsx
+++ b/data/assumptions_register.xlsx
@@ -71,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -95,6 +95,12 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -486,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -548,7 +554,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>re_target_2030</t>
         </is>
@@ -558,15 +564,15 @@
           <t>Renewable share of electricity generation, 2030</t>
         </is>
       </c>
-      <c r="C2" s="18" t="n">
+      <c r="C2" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="D2" s="17" t="inlineStr">
+      <c r="D2" s="19" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E2" s="17" t="inlineStr">
+      <c r="E2" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -576,12 +582,12 @@
           <t>TAP, 9 Oct 2026: Head of Government reaffirms 35% target</t>
         </is>
       </c>
-      <c r="G2" s="17" t="inlineStr">
+      <c r="G2" s="19" t="inlineStr">
         <is>
           <t>https://www.tap.info.tn/fr/Portail-%C3%A0-la-Une-FR-top/20672933-%C3%A9nergie-la</t>
         </is>
       </c>
-      <c r="H2" s="17" t="inlineStr">
+      <c r="H2" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -593,7 +599,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>flex_cap_mw</t>
         </is>
@@ -603,15 +609,15 @@
           <t>Shiftable load cap (scenario S2-300)</t>
         </is>
       </c>
-      <c r="C3" s="18" t="n">
+      <c r="C3" s="20" t="n">
         <v>300</v>
       </c>
-      <c r="D3" s="17" t="inlineStr">
+      <c r="D3" s="19" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E3" s="17" t="inlineStr">
+      <c r="E3" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -621,12 +627,12 @@
           <t>TAP, 9 Oct 2026: action plan targets 300 MW peak-demand reduction</t>
         </is>
       </c>
-      <c r="G3" s="17" t="inlineStr">
+      <c r="G3" s="19" t="inlineStr">
         <is>
           <t>https://www.tap.info.tn/fr/Portail-%C3%A0-la-Une-FR-top/20672933-%C3%A9nergie-la</t>
         </is>
       </c>
-      <c r="H3" s="17" t="inlineStr">
+      <c r="H3" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -638,7 +644,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>flex_cap_hi_mw</t>
         </is>
@@ -648,22 +654,22 @@
           <t>Shiftable load cap, sensitivity (S2-600)</t>
         </is>
       </c>
-      <c r="C4" s="18" t="n">
+      <c r="C4" s="20" t="n">
         <v>600</v>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="19" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="17" t="inlineStr"/>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="G4" s="19" t="inlineStr"/>
+      <c r="H4" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -675,7 +681,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>flex_max_hours</t>
         </is>
@@ -685,22 +691,22 @@
           <t>Maximum shift duration</t>
         </is>
       </c>
-      <c r="C5" s="18" t="n">
+      <c r="C5" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="17" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="17" t="inlineStr"/>
-      <c r="H5" s="17" t="inlineStr">
+      <c r="G5" s="19" t="inlineStr"/>
+      <c r="H5" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -712,7 +718,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>gas_price_factor_lo</t>
         </is>
@@ -722,22 +728,22 @@
           <t>Gas price sensitivity, low</t>
         </is>
       </c>
-      <c r="C6" s="18" t="n">
+      <c r="C6" s="20" t="n">
         <v>0.5</v>
       </c>
-      <c r="D6" s="17" t="inlineStr">
+      <c r="D6" s="19" t="inlineStr">
         <is>
           <t>x base</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="E6" s="19" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="17" t="inlineStr"/>
-      <c r="H6" s="17" t="inlineStr">
+      <c r="G6" s="19" t="inlineStr"/>
+      <c r="H6" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -749,7 +755,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>gas_price_factor_hi</t>
         </is>
@@ -759,22 +765,22 @@
           <t>Gas price sensitivity, high</t>
         </is>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7" s="20" t="n">
         <v>1.5</v>
       </c>
-      <c r="D7" s="17" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>x base</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="17" t="inlineStr"/>
-      <c r="H7" s="17" t="inlineStr">
+      <c r="G7" s="19" t="inlineStr"/>
+      <c r="H7" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -786,25 +792,25 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>demand_growth</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Electricity demand growth 2022-2030 (CAGR)</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="n">
+          <t>Electricity demand growth rate (STEG base case, applied 2024 -&gt; 2030)</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="n">
         <v>0.032</v>
       </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="D8" s="19" t="inlineStr">
         <is>
           <t>1/yr</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -814,12 +820,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.2-17 and p.5-34</t>
         </is>
       </c>
-      <c r="G8" s="17" t="inlineStr">
+      <c r="G8" s="19" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H8" s="17" t="inlineStr">
+      <c r="H8" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -831,7 +837,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>peak_ref_2030_mw</t>
         </is>
@@ -841,15 +847,15 @@
           <t>Reference 2030 peak demand</t>
         </is>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="20" t="n">
         <v>6000</v>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -859,12 +865,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.2-17 and p.5-35</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
+      <c r="G9" s="19" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="H9" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -876,7 +882,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>discount_rate</t>
         </is>
@@ -886,15 +892,15 @@
           <t>Discount rate for annualising investment</t>
         </is>
       </c>
-      <c r="C10" s="18" t="n">
+      <c r="C10" s="20" t="n">
         <v>0.07099999999999999</v>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>1/yr</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr">
+      <c r="E10" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -904,12 +910,12 @@
           <t>PyPSA-Earth v0.10.0 config.default.yaml, costs.discountrate</t>
         </is>
       </c>
-      <c r="G10" s="17" t="inlineStr">
+      <c r="G10" s="19" t="inlineStr">
         <is>
           <t>https://github.com/pypsa-meets-earth/pypsa-earth/blob/v0.10.0/config.default.yaml</t>
         </is>
       </c>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="H10" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -921,7 +927,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>demand_2024_twh</t>
         </is>
@@ -931,15 +937,15 @@
           <t>Electricity demand 2024 (generation + net imports)</t>
         </is>
       </c>
-      <c r="C11" s="18" t="n">
+      <c r="C11" s="20" t="n">
         <v>22.507</v>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E11" s="17" t="inlineStr">
+      <c r="E11" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -949,12 +955,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025), table 'ELECTRICITE', printed p.18</t>
         </is>
       </c>
-      <c r="G11" s="17" t="inlineStr">
+      <c r="G11" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="H11" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -966,7 +972,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>imports_2024_twh</t>
         </is>
@@ -976,15 +982,15 @@
           <t>Net electricity imports 2024</t>
         </is>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="20" t="n">
         <v>3.1131</v>
       </c>
-      <c r="D12" s="17" t="inlineStr">
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E12" s="17" t="inlineStr">
+      <c r="E12" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -994,12 +1000,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025), table 'ELECTRICITE', printed p.18</t>
         </is>
       </c>
-      <c r="G12" s="17" t="inlineStr">
+      <c r="G12" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H12" s="17" t="inlineStr">
+      <c r="H12" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -1011,7 +1017,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>gas_price_eur_per_mwh_th</t>
         </is>
@@ -1021,15 +1027,15 @@
           <t>Natural gas price (economic cost)</t>
         </is>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="C13" s="20" t="n">
         <v>28.4158</v>
       </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>EUR/MWh_th</t>
         </is>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="E13" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1039,12 +1045,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, fuel); original: World Bank Commodity Markets 2025 and ENTSO-E/ENTSOG TYNDP 2024</t>
         </is>
       </c>
-      <c r="G13" s="17" t="inlineStr">
+      <c r="G13" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H13" s="17" t="inlineStr">
+      <c r="H13" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -1056,7 +1062,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>toy_ccgt_investment</t>
         </is>
@@ -1066,15 +1072,15 @@
           <t>CCGT investment</t>
         </is>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="20" t="n">
         <v>1108.7166</v>
       </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>EUR/kW</t>
         </is>
       </c>
-      <c r="E14" s="17" t="inlineStr">
+      <c r="E14" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1084,12 +1090,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G14" s="17" t="inlineStr">
+      <c r="G14" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H14" s="17" t="inlineStr">
+      <c r="H14" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1101,7 +1107,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>toy_ccgt_fom</t>
         </is>
@@ -1111,15 +1117,15 @@
           <t>CCGT fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C15" s="18" t="n">
+      <c r="C15" s="20" t="n">
         <v>3.3494</v>
       </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E15" s="17" t="inlineStr">
+      <c r="E15" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1129,12 +1135,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G15" s="17" t="inlineStr">
+      <c r="G15" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H15" s="17" t="inlineStr">
+      <c r="H15" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1146,7 +1152,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>toy_ccgt_vom</t>
         </is>
@@ -1156,15 +1162,15 @@
           <t>CCGT variable O&amp;M</t>
         </is>
       </c>
-      <c r="C16" s="18" t="n">
+      <c r="C16" s="20" t="n">
         <v>5.6104</v>
       </c>
-      <c r="D16" s="17" t="inlineStr">
+      <c r="D16" s="19" t="inlineStr">
         <is>
           <t>EUR/MWh</t>
         </is>
       </c>
-      <c r="E16" s="17" t="inlineStr">
+      <c r="E16" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1174,12 +1180,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G16" s="17" t="inlineStr">
+      <c r="G16" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H16" s="17" t="inlineStr">
+      <c r="H16" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1191,7 +1197,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>toy_ccgt_efficiency</t>
         </is>
@@ -1201,15 +1207,15 @@
           <t>CCGT electrical efficiency</t>
         </is>
       </c>
-      <c r="C17" s="18" t="n">
+      <c r="C17" s="20" t="n">
         <v>0.58</v>
       </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>per unit</t>
         </is>
       </c>
-      <c r="E17" s="17" t="inlineStr">
+      <c r="E17" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1219,12 +1225,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, efficiency); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G17" s="17" t="inlineStr">
+      <c r="G17" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H17" s="17" t="inlineStr">
+      <c r="H17" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1236,7 +1242,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>toy_ccgt_lifetime</t>
         </is>
@@ -1246,15 +1252,15 @@
           <t>CCGT lifetime</t>
         </is>
       </c>
-      <c r="C18" s="18" t="n">
+      <c r="C18" s="20" t="n">
         <v>25</v>
       </c>
-      <c r="D18" s="17" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E18" s="17" t="inlineStr">
+      <c r="E18" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1264,12 +1270,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G18" s="17" t="inlineStr">
+      <c r="G18" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H18" s="17" t="inlineStr">
+      <c r="H18" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1281,7 +1287,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>toy_solar_investment</t>
         </is>
@@ -1291,15 +1297,15 @@
           <t>Utility PV investment</t>
         </is>
       </c>
-      <c r="C19" s="18" t="n">
+      <c r="C19" s="20" t="n">
         <v>482.4785</v>
       </c>
-      <c r="D19" s="17" t="inlineStr">
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>EUR/kW_e</t>
         </is>
       </c>
-      <c r="E19" s="17" t="inlineStr">
+      <c r="E19" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1309,12 +1315,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G19" s="17" t="inlineStr">
+      <c r="G19" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H19" s="17" t="inlineStr">
+      <c r="H19" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1326,7 +1332,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>toy_solar_fom</t>
         </is>
@@ -1336,15 +1342,15 @@
           <t>Utility PV fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C20" s="18" t="n">
+      <c r="C20" s="20" t="n">
         <v>2.4757</v>
       </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E20" s="17" t="inlineStr">
+      <c r="E20" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1354,12 +1360,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G20" s="17" t="inlineStr">
+      <c r="G20" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H20" s="17" t="inlineStr">
+      <c r="H20" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1371,7 +1377,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>toy_solar_lifetime</t>
         </is>
@@ -1381,15 +1387,15 @@
           <t>Utility PV lifetime</t>
         </is>
       </c>
-      <c r="C21" s="18" t="n">
+      <c r="C21" s="20" t="n">
         <v>40</v>
       </c>
-      <c r="D21" s="17" t="inlineStr">
+      <c r="D21" s="19" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E21" s="17" t="inlineStr">
+      <c r="E21" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1399,12 +1405,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G21" s="17" t="inlineStr">
+      <c r="G21" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H21" s="17" t="inlineStr">
+      <c r="H21" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1416,7 +1422,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>toy_onwind_investment</t>
         </is>
@@ -1426,15 +1432,15 @@
           <t>Onshore wind investment</t>
         </is>
       </c>
-      <c r="C22" s="18" t="n">
+      <c r="C22" s="20" t="n">
         <v>1383.3059</v>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D22" s="19" t="inlineStr">
         <is>
           <t>EUR/kW</t>
         </is>
       </c>
-      <c r="E22" s="17" t="inlineStr">
+      <c r="E22" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1444,12 +1450,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G22" s="17" t="inlineStr">
+      <c r="G22" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H22" s="17" t="inlineStr">
+      <c r="H22" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1461,7 +1467,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>toy_onwind_fom</t>
         </is>
@@ -1471,15 +1477,15 @@
           <t>Onshore wind fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C23" s="18" t="n">
+      <c r="C23" s="20" t="n">
         <v>1.2167</v>
       </c>
-      <c r="D23" s="17" t="inlineStr">
+      <c r="D23" s="19" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E23" s="17" t="inlineStr">
+      <c r="E23" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1489,12 +1495,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G23" s="17" t="inlineStr">
+      <c r="G23" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H23" s="17" t="inlineStr">
+      <c r="H23" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1506,7 +1512,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>toy_onwind_vom</t>
         </is>
@@ -1516,15 +1522,15 @@
           <t>Onshore wind variable O&amp;M</t>
         </is>
       </c>
-      <c r="C24" s="18" t="n">
+      <c r="C24" s="20" t="n">
         <v>1.8033</v>
       </c>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
         <is>
           <t>EUR/MWh</t>
         </is>
       </c>
-      <c r="E24" s="17" t="inlineStr">
+      <c r="E24" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1534,12 +1540,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G24" s="17" t="inlineStr">
+      <c r="G24" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H24" s="17" t="inlineStr">
+      <c r="H24" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1551,7 +1557,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>toy_onwind_lifetime</t>
         </is>
@@ -1561,15 +1567,15 @@
           <t>Onshore wind lifetime</t>
         </is>
       </c>
-      <c r="C25" s="18" t="n">
+      <c r="C25" s="20" t="n">
         <v>30</v>
       </c>
-      <c r="D25" s="17" t="inlineStr">
+      <c r="D25" s="19" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E25" s="17" t="inlineStr">
+      <c r="E25" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1579,12 +1585,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G25" s="17" t="inlineStr">
+      <c r="G25" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H25" s="17" t="inlineStr">
+      <c r="H25" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1596,7 +1602,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="inlineStr">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>toy_battery_storage_investment</t>
         </is>
@@ -1606,15 +1612,15 @@
           <t>Battery energy (storage) investment</t>
         </is>
       </c>
-      <c r="C26" s="18" t="n">
+      <c r="C26" s="20" t="n">
         <v>189.861</v>
       </c>
-      <c r="D26" s="17" t="inlineStr">
+      <c r="D26" s="19" t="inlineStr">
         <is>
           <t>EUR/kWh</t>
         </is>
       </c>
-      <c r="E26" s="17" t="inlineStr">
+      <c r="E26" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1624,12 +1630,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery storage, investment); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G26" s="17" t="inlineStr">
+      <c r="G26" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H26" s="17" t="inlineStr">
+      <c r="H26" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1641,7 +1647,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>toy_battery_storage_lifetime</t>
         </is>
@@ -1651,15 +1657,15 @@
           <t>Battery energy (storage) lifetime</t>
         </is>
       </c>
-      <c r="C27" s="18" t="n">
+      <c r="C27" s="20" t="n">
         <v>25</v>
       </c>
-      <c r="D27" s="17" t="inlineStr">
+      <c r="D27" s="19" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E27" s="17" t="inlineStr">
+      <c r="E27" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1669,12 +1675,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery storage, lifetime); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G27" s="17" t="inlineStr">
+      <c r="G27" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H27" s="17" t="inlineStr">
+      <c r="H27" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1686,7 +1692,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="inlineStr">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>toy_battery_inverter_investment</t>
         </is>
@@ -1696,15 +1702,15 @@
           <t>Battery inverter (power) investment</t>
         </is>
       </c>
-      <c r="C28" s="18" t="n">
+      <c r="C28" s="20" t="n">
         <v>213.9279</v>
       </c>
-      <c r="D28" s="17" t="inlineStr">
+      <c r="D28" s="19" t="inlineStr">
         <is>
           <t>EUR/kW</t>
         </is>
       </c>
-      <c r="E28" s="17" t="inlineStr">
+      <c r="E28" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1714,12 +1720,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, investment); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G28" s="17" t="inlineStr">
+      <c r="G28" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H28" s="17" t="inlineStr">
+      <c r="H28" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1731,7 +1737,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="inlineStr">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>toy_battery_inverter_fom</t>
         </is>
@@ -1741,15 +1747,15 @@
           <t>Battery inverter fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C29" s="18" t="n">
+      <c r="C29" s="20" t="n">
         <v>0.3375</v>
       </c>
-      <c r="D29" s="17" t="inlineStr">
+      <c r="D29" s="19" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E29" s="17" t="inlineStr">
+      <c r="E29" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1759,12 +1765,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, FOM); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G29" s="17" t="inlineStr">
+      <c r="G29" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H29" s="17" t="inlineStr">
+      <c r="H29" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1776,7 +1782,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="inlineStr">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>toy_battery_inverter_efficiency</t>
         </is>
@@ -1786,15 +1792,15 @@
           <t>Battery round-trip efficiency (source: 'Round trip efficiency DC')</t>
         </is>
       </c>
-      <c r="C30" s="18" t="n">
+      <c r="C30" s="20" t="n">
         <v>0.96</v>
       </c>
-      <c r="D30" s="17" t="inlineStr">
+      <c r="D30" s="19" t="inlineStr">
         <is>
           <t>per unit</t>
         </is>
       </c>
-      <c r="E30" s="17" t="inlineStr">
+      <c r="E30" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1804,12 +1810,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, efficiency); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G30" s="17" t="inlineStr">
+      <c r="G30" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H30" s="17" t="inlineStr">
+      <c r="H30" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1821,7 +1827,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="inlineStr">
+      <c r="A31" s="19" t="inlineStr">
         <is>
           <t>toy_battery_inverter_lifetime</t>
         </is>
@@ -1831,15 +1837,15 @@
           <t>Battery inverter lifetime</t>
         </is>
       </c>
-      <c r="C31" s="18" t="n">
+      <c r="C31" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="D31" s="17" t="inlineStr">
+      <c r="D31" s="19" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E31" s="17" t="inlineStr">
+      <c r="E31" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1849,12 +1855,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, lifetime); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx, Note K.</t>
         </is>
       </c>
-      <c r="G31" s="17" t="inlineStr">
+      <c r="G31" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H31" s="17" t="inlineStr">
+      <c r="H31" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1866,7 +1872,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="17" t="inlineStr">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>toy_gas_fuel</t>
         </is>
@@ -1876,15 +1882,15 @@
           <t>Natural gas fuel cost</t>
         </is>
       </c>
-      <c r="C32" s="18" t="n">
+      <c r="C32" s="20" t="n">
         <v>28.4158</v>
       </c>
-      <c r="D32" s="17" t="inlineStr">
+      <c r="D32" s="19" t="inlineStr">
         <is>
           <t>EUR/MWh_th</t>
         </is>
       </c>
-      <c r="E32" s="17" t="inlineStr">
+      <c r="E32" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1894,12 +1900,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, fuel); original: World Bank (2025) Commodity Markets, https://www.worldbank.org/en/research/commodity-markets; and ENTSO-E &amp; ENTSOG TYNDP 2024 Scenarios Inputs Commodity Prices, https://2024-data.entsos-tyndp-scenarios.eu/files/scenarios-inputs/Prices.zip, accessed: 2026-02-03.</t>
         </is>
       </c>
-      <c r="G32" s="17" t="inlineStr">
+      <c r="G32" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H32" s="17" t="inlineStr">
+      <c r="H32" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1911,7 +1917,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>toy_gas_co2_intensity</t>
         </is>
@@ -1921,15 +1927,15 @@
           <t>Natural gas CO2 intensity</t>
         </is>
       </c>
-      <c r="C33" s="18" t="n">
+      <c r="C33" s="20" t="n">
         <v>0.198</v>
       </c>
-      <c r="D33" s="17" t="inlineStr">
+      <c r="D33" s="19" t="inlineStr">
         <is>
           <t>tCO2/MWh_th</t>
         </is>
       </c>
-      <c r="E33" s="17" t="inlineStr">
+      <c r="E33" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1939,12 +1945,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, CO2 intensity); original: Stoichiometric calculation with 50 GJ/t CH4</t>
         </is>
       </c>
-      <c r="G33" s="17" t="inlineStr">
+      <c r="G33" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H33" s="17" t="inlineStr">
+      <c r="H33" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1956,7 +1962,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="17" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>toy_battery_max_hours</t>
         </is>
@@ -1966,22 +1972,22 @@
           <t>Toy battery energy-to-power ratio</t>
         </is>
       </c>
-      <c r="C34" s="18" t="n">
+      <c r="C34" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="D34" s="17" t="inlineStr">
+      <c r="D34" s="19" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="E34" s="17" t="inlineStr">
+      <c r="E34" s="19" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr"/>
-      <c r="G34" s="17" t="inlineStr"/>
-      <c r="H34" s="17" t="inlineStr">
+      <c r="G34" s="19" t="inlineStr"/>
+      <c r="H34" s="19" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1993,7 +1999,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="inlineStr">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>cap_2024_ccgt_mw</t>
         </is>
@@ -2003,15 +2009,15 @@
           <t>Net installed capacity 2024: combined cycle</t>
         </is>
       </c>
-      <c r="C35" s="18" t="n">
+      <c r="C35" s="20" t="n">
         <v>2527</v>
       </c>
-      <c r="D35" s="17" t="inlineStr">
+      <c r="D35" s="19" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E35" s="17" t="inlineStr">
+      <c r="E35" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2021,12 +2027,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G35" s="17" t="inlineStr">
+      <c r="G35" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H35" s="17" t="inlineStr">
+      <c r="H35" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2038,7 +2044,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="17" t="inlineStr">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>cap_2024_ocgt_mw</t>
         </is>
@@ -2048,15 +2054,15 @@
           <t>Net installed capacity 2024: gas turbines (open cycle)</t>
         </is>
       </c>
-      <c r="C36" s="18" t="n">
+      <c r="C36" s="20" t="n">
         <v>2457</v>
       </c>
-      <c r="D36" s="17" t="inlineStr">
+      <c r="D36" s="19" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E36" s="17" t="inlineStr">
+      <c r="E36" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2066,12 +2072,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G36" s="17" t="inlineStr">
+      <c r="G36" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H36" s="17" t="inlineStr">
+      <c r="H36" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2083,7 +2089,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="inlineStr">
+      <c r="A37" s="19" t="inlineStr">
         <is>
           <t>cap_2024_steam_mw</t>
         </is>
@@ -2093,15 +2099,15 @@
           <t>Net installed capacity 2024: steam turbines</t>
         </is>
       </c>
-      <c r="C37" s="18" t="n">
+      <c r="C37" s="20" t="n">
         <v>660</v>
       </c>
-      <c r="D37" s="17" t="inlineStr">
+      <c r="D37" s="19" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E37" s="17" t="inlineStr">
+      <c r="E37" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2111,12 +2117,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G37" s="17" t="inlineStr">
+      <c r="G37" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H37" s="17" t="inlineStr">
+      <c r="H37" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2128,7 +2134,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="inlineStr">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>cap_2024_re_mw</t>
         </is>
@@ -2138,15 +2144,15 @@
           <t>Net installed capacity 2024: renewables (hydro + wind + solar, centralised)</t>
         </is>
       </c>
-      <c r="C38" s="18" t="n">
+      <c r="C38" s="20" t="n">
         <v>368</v>
       </c>
-      <c r="D38" s="17" t="inlineStr">
+      <c r="D38" s="19" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E38" s="17" t="inlineStr">
+      <c r="E38" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2156,12 +2162,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G38" s="17" t="inlineStr">
+      <c r="G38" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H38" s="17" t="inlineStr">
+      <c r="H38" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2173,7 +2179,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="17" t="inlineStr">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t>cap_2024_total_mw</t>
         </is>
@@ -2183,15 +2189,15 @@
           <t>Net installed capacity 2024: total</t>
         </is>
       </c>
-      <c r="C39" s="18" t="n">
+      <c r="C39" s="20" t="n">
         <v>6012</v>
       </c>
-      <c r="D39" s="17" t="inlineStr">
+      <c r="D39" s="19" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E39" s="17" t="inlineStr">
+      <c r="E39" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2201,12 +2207,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G39" s="17" t="inlineStr">
+      <c r="G39" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H39" s="17" t="inlineStr">
+      <c r="H39" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2218,7 +2224,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="17" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr">
         <is>
           <t>gen_2024_gas_twh</t>
         </is>
@@ -2228,15 +2234,15 @@
           <t>Electricity generation 2024: natural gas</t>
         </is>
       </c>
-      <c r="C40" s="18" t="n">
+      <c r="C40" s="20" t="n">
         <v>18.156</v>
       </c>
-      <c r="D40" s="17" t="inlineStr">
+      <c r="D40" s="19" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E40" s="17" t="inlineStr">
+      <c r="E40" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2246,12 +2252,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G40" s="17" t="inlineStr">
+      <c r="G40" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H40" s="17" t="inlineStr">
+      <c r="H40" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2263,7 +2269,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="17" t="inlineStr">
+      <c r="A41" s="19" t="inlineStr">
         <is>
           <t>gen_2024_oil_twh</t>
         </is>
@@ -2273,15 +2279,15 @@
           <t>Electricity generation 2024: fuel oil + gasoil</t>
         </is>
       </c>
-      <c r="C41" s="18" t="n">
+      <c r="C41" s="20" t="n">
         <v>0.07190000000000001</v>
       </c>
-      <c r="D41" s="17" t="inlineStr">
+      <c r="D41" s="19" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E41" s="17" t="inlineStr">
+      <c r="E41" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2291,12 +2297,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G41" s="17" t="inlineStr">
+      <c r="G41" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H41" s="17" t="inlineStr">
+      <c r="H41" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2308,7 +2314,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="17" t="inlineStr">
+      <c r="A42" s="19" t="inlineStr">
         <is>
           <t>gen_2024_hydro_twh</t>
         </is>
@@ -2318,15 +2324,15 @@
           <t>Electricity generation 2024: hydro</t>
         </is>
       </c>
-      <c r="C42" s="18" t="n">
+      <c r="C42" s="20" t="n">
         <v>0.016</v>
       </c>
-      <c r="D42" s="17" t="inlineStr">
+      <c r="D42" s="19" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E42" s="17" t="inlineStr">
+      <c r="E42" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2336,12 +2342,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G42" s="17" t="inlineStr">
+      <c r="G42" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H42" s="17" t="inlineStr">
+      <c r="H42" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2353,7 +2359,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="17" t="inlineStr">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t>gen_2024_wind_twh</t>
         </is>
@@ -2363,15 +2369,15 @@
           <t>Electricity generation 2024: wind</t>
         </is>
       </c>
-      <c r="C43" s="18" t="n">
+      <c r="C43" s="20" t="n">
         <v>0.337</v>
       </c>
-      <c r="D43" s="17" t="inlineStr">
+      <c r="D43" s="19" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E43" s="17" t="inlineStr">
+      <c r="E43" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2381,12 +2387,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G43" s="17" t="inlineStr">
+      <c r="G43" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H43" s="17" t="inlineStr">
+      <c r="H43" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2398,7 +2404,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="inlineStr">
+      <c r="A44" s="19" t="inlineStr">
         <is>
           <t>gen_2024_solar_twh</t>
         </is>
@@ -2408,15 +2414,15 @@
           <t>Electricity generation 2024: solar PV (STEG + IPP + self-generation)</t>
         </is>
       </c>
-      <c r="C44" s="18" t="n">
+      <c r="C44" s="20" t="n">
         <v>0.6278</v>
       </c>
-      <c r="D44" s="17" t="inlineStr">
+      <c r="D44" s="19" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E44" s="17" t="inlineStr">
+      <c r="E44" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2426,12 +2432,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G44" s="17" t="inlineStr">
+      <c r="G44" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H44" s="17" t="inlineStr">
+      <c r="H44" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2443,7 +2449,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="17" t="inlineStr">
+      <c r="A45" s="19" t="inlineStr">
         <is>
           <t>gen_2024_total_twh</t>
         </is>
@@ -2453,15 +2459,15 @@
           <t>Electricity generation 2024: total</t>
         </is>
       </c>
-      <c r="C45" s="18" t="n">
+      <c r="C45" s="20" t="n">
         <v>19.208</v>
       </c>
-      <c r="D45" s="17" t="inlineStr">
+      <c r="D45" s="19" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E45" s="17" t="inlineStr">
+      <c r="E45" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2471,12 +2477,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G45" s="17" t="inlineStr">
+      <c r="G45" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H45" s="17" t="inlineStr">
+      <c r="H45" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2488,7 +2494,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="17" t="inlineStr">
+      <c r="A46" s="19" t="inlineStr">
         <is>
           <t>gas_share_2024</t>
         </is>
@@ -2498,15 +2504,15 @@
           <t>Gas share of electricity generation 2024</t>
         </is>
       </c>
-      <c r="C46" s="18" t="n">
+      <c r="C46" s="20" t="n">
         <v>0.945</v>
       </c>
-      <c r="D46" s="17" t="inlineStr">
+      <c r="D46" s="19" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E46" s="17" t="inlineStr">
+      <c r="E46" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2516,12 +2522,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G46" s="17" t="inlineStr">
+      <c r="G46" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H46" s="17" t="inlineStr">
+      <c r="H46" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2533,7 +2539,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="17" t="inlineStr">
+      <c r="A47" s="19" t="inlineStr">
         <is>
           <t>peak_2024_mw</t>
         </is>
@@ -2543,15 +2549,15 @@
           <t>Peak electricity demand 2024</t>
         </is>
       </c>
-      <c r="C47" s="18" t="n">
+      <c r="C47" s="20" t="n">
         <v>4888</v>
       </c>
-      <c r="D47" s="17" t="inlineStr">
+      <c r="D47" s="19" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E47" s="17" t="inlineStr">
+      <c r="E47" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2561,12 +2567,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G47" s="17" t="inlineStr">
+      <c r="G47" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H47" s="17" t="inlineStr">
+      <c r="H47" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2578,7 +2584,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="17" t="inlineStr">
+      <c r="A48" s="19" t="inlineStr">
         <is>
           <t>steg_specific_consumption_2024</t>
         </is>
@@ -2588,15 +2594,15 @@
           <t>STEG fleet specific fuel consumption 2024</t>
         </is>
       </c>
-      <c r="C48" s="18" t="n">
+      <c r="C48" s="20" t="n">
         <v>194.8</v>
       </c>
-      <c r="D48" s="17" t="inlineStr">
+      <c r="D48" s="19" t="inlineStr">
         <is>
           <t>toe(GCV)/GWh</t>
         </is>
       </c>
-      <c r="E48" s="17" t="inlineStr">
+      <c r="E48" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2606,12 +2612,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G48" s="17" t="inlineStr">
+      <c r="G48" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H48" s="17" t="inlineStr">
+      <c r="H48" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2623,7 +2629,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="17" t="inlineStr">
+      <c r="A49" s="19" t="inlineStr">
         <is>
           <t>steg_demand_2030_gwh</t>
         </is>
@@ -2633,15 +2639,15 @@
           <t>STEG forecast of 2030 electricity demand</t>
         </is>
       </c>
-      <c r="C49" s="18" t="n">
+      <c r="C49" s="20" t="n">
         <v>28362</v>
       </c>
-      <c r="D49" s="17" t="inlineStr">
+      <c r="D49" s="19" t="inlineStr">
         <is>
           <t>GWh</t>
         </is>
       </c>
-      <c r="E49" s="17" t="inlineStr">
+      <c r="E49" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2651,12 +2657,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.2-17</t>
         </is>
       </c>
-      <c r="G49" s="17" t="inlineStr">
+      <c r="G49" s="19" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H49" s="17" t="inlineStr">
+      <c r="H49" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2668,7 +2674,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="17" t="inlineStr">
+      <c r="A50" s="19" t="inlineStr">
         <is>
           <t>load_factor_2030</t>
         </is>
@@ -2678,15 +2684,15 @@
           <t>STEG 2030 forecast: annual load factor</t>
         </is>
       </c>
-      <c r="C50" s="18" t="n">
+      <c r="C50" s="20" t="n">
         <v>0.54</v>
       </c>
-      <c r="D50" s="17" t="inlineStr">
+      <c r="D50" s="19" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E50" s="17" t="inlineStr">
+      <c r="E50" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2696,12 +2702,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.5-34</t>
         </is>
       </c>
-      <c r="G50" s="17" t="inlineStr">
+      <c r="G50" s="19" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H50" s="17" t="inlineStr">
+      <c r="H50" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2713,7 +2719,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="17" t="inlineStr">
+      <c r="A51" s="19" t="inlineStr">
         <is>
           <t>min_to_peak_2030</t>
         </is>
@@ -2723,15 +2729,15 @@
           <t>STEG 2030 forecast: minimum-to-peak load ratio</t>
         </is>
       </c>
-      <c r="C51" s="18" t="n">
+      <c r="C51" s="20" t="n">
         <v>0.34</v>
       </c>
-      <c r="D51" s="17" t="inlineStr">
+      <c r="D51" s="19" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E51" s="17" t="inlineStr">
+      <c r="E51" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2741,12 +2747,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.5-35</t>
         </is>
       </c>
-      <c r="G51" s="17" t="inlineStr">
+      <c r="G51" s="19" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H51" s="17" t="inlineStr">
+      <c r="H51" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2758,7 +2764,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="17" t="inlineStr">
+      <c r="A52" s="19" t="inlineStr">
         <is>
           <t>ccgt_efficiency</t>
         </is>
@@ -2768,15 +2774,15 @@
           <t>CCGT electrical efficiency (new build)</t>
         </is>
       </c>
-      <c r="C52" s="18" t="n">
+      <c r="C52" s="20" t="n">
         <v>0.58</v>
       </c>
-      <c r="D52" s="17" t="inlineStr">
+      <c r="D52" s="19" t="inlineStr">
         <is>
           <t>per unit</t>
         </is>
       </c>
-      <c r="E52" s="17" t="inlineStr">
+      <c r="E52" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2786,12 +2792,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, efficiency); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G52" s="17" t="inlineStr">
+      <c r="G52" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H52" s="17" t="inlineStr">
+      <c r="H52" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2803,7 +2809,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="17" t="inlineStr">
+      <c r="A53" s="19" t="inlineStr">
         <is>
           <t>ccgt_vom</t>
         </is>
@@ -2813,15 +2819,15 @@
           <t>CCGT variable O&amp;M</t>
         </is>
       </c>
-      <c r="C53" s="18" t="n">
+      <c r="C53" s="20" t="n">
         <v>5.6104</v>
       </c>
-      <c r="D53" s="17" t="inlineStr">
+      <c r="D53" s="19" t="inlineStr">
         <is>
           <t>EUR/MWh</t>
         </is>
       </c>
-      <c r="E53" s="17" t="inlineStr">
+      <c r="E53" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2831,12 +2837,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G53" s="17" t="inlineStr">
+      <c r="G53" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H53" s="17" t="inlineStr">
+      <c r="H53" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2848,7 +2854,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="17" t="inlineStr">
+      <c r="A54" s="19" t="inlineStr">
         <is>
           <t>ocgt_efficiency</t>
         </is>
@@ -2858,15 +2864,15 @@
           <t>OCGT electrical efficiency (new build)</t>
         </is>
       </c>
-      <c r="C54" s="18" t="n">
+      <c r="C54" s="20" t="n">
         <v>0.41</v>
       </c>
-      <c r="D54" s="17" t="inlineStr">
+      <c r="D54" s="19" t="inlineStr">
         <is>
           <t>per unit</t>
         </is>
       </c>
-      <c r="E54" s="17" t="inlineStr">
+      <c r="E54" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2876,12 +2882,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (OCGT, efficiency); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G54" s="17" t="inlineStr">
+      <c r="G54" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H54" s="17" t="inlineStr">
+      <c r="H54" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2893,7 +2899,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="17" t="inlineStr">
+      <c r="A55" s="19" t="inlineStr">
         <is>
           <t>ocgt_vom</t>
         </is>
@@ -2903,15 +2909,15 @@
           <t>OCGT variable O&amp;M</t>
         </is>
       </c>
-      <c r="C55" s="18" t="n">
+      <c r="C55" s="20" t="n">
         <v>6.0111</v>
       </c>
-      <c r="D55" s="17" t="inlineStr">
+      <c r="D55" s="19" t="inlineStr">
         <is>
           <t>EUR/MWh</t>
         </is>
       </c>
-      <c r="E55" s="17" t="inlineStr">
+      <c r="E55" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2921,12 +2927,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (OCGT, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G55" s="17" t="inlineStr">
+      <c r="G55" s="19" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H55" s="17" t="inlineStr">
+      <c r="H55" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2938,7 +2944,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="17" t="inlineStr">
+      <c r="A56" s="19" t="inlineStr">
         <is>
           <t>gas_ncv_per_gcv</t>
         </is>
@@ -2948,15 +2954,15 @@
           <t>Natural gas: net / gross calorific value</t>
         </is>
       </c>
-      <c r="C56" s="18" t="n">
+      <c r="C56" s="20" t="n">
         <v>0.9</v>
       </c>
-      <c r="D56" s="17" t="inlineStr">
+      <c r="D56" s="19" t="inlineStr">
         <is>
           <t>ratio</t>
         </is>
       </c>
-      <c r="E56" s="17" t="inlineStr">
+      <c r="E56" s="19" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2966,12 +2972,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024, conversion table (PDF p.22)</t>
         </is>
       </c>
-      <c r="G56" s="17" t="inlineStr">
+      <c r="G56" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H56" s="17" t="inlineStr">
+      <c r="H56" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2983,7 +2989,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="17" t="inlineStr">
+      <c r="A57" s="19" t="inlineStr">
         <is>
           <t>existing_gas_efficiency_factor</t>
         </is>
@@ -2993,17 +2999,17 @@
           <t>Efficiency factor for existing gas units (calibrated)</t>
         </is>
       </c>
-      <c r="C57" s="18" t="n">
+      <c r="C57" s="20" t="n">
         <v>0.8633999999999999</v>
       </c>
-      <c r="D57" s="17" t="inlineStr">
+      <c r="D57" s="19" t="inlineStr">
         <is>
           <t>x tech-data</t>
         </is>
       </c>
-      <c r="E57" s="17" t="inlineStr">
-        <is>
-          <t>sourced</t>
+      <c r="E57" s="19" t="inlineStr">
+        <is>
+          <t>assumption</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -3011,19 +3017,334 @@
           <t>Calibrated (Task 10) so the dispatch-only 2024 run matches STEG's measured fuel use: ONEM Memento 2024, specific consumption 194.8 toe(PCS)/GWh, PCI = 0.9 PCS</t>
         </is>
       </c>
-      <c r="G57" s="17" t="inlineStr">
+      <c r="G57" s="19" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H57" s="17" t="inlineStr">
+      <c r="H57" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>Computed by scripts/validate_baseline.py: target fleet efficiency 0.490 (net) / model 0.568 at factor 1. Existing CCGT 0.58 x 0.8634 = 0.501; existing OCGT + steam 0.41 x 0.8634 = 0.354. New builds keep tech-data values.</t>
+          <t>Calibration, not a published figure. Fitted by scripts/validate_baseline.py so the 2024 dispatch-only run matches STEG's measured fuel use (ONEM Memento 2024: 194.8 toe(PCS)/GWh; PCI = 0.9 PCS). Target 0.490 (net) / model 0.568 at factor 1. Existing CCGT 0.58 x 0.8634 = 0.501; existing OCGT + steam 0.41 x 0.8634 = 0.354. Also absorbs unmodelled outages and part-load operation (the model has no availability limits). New builds keep tech-data values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="19" t="inlineStr">
+        <is>
+          <t>ocgt_investment</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>OCGT investment (new build)</t>
+        </is>
+      </c>
+      <c r="C58" s="20" t="n">
+        <v>581.3949</v>
+      </c>
+      <c r="D58" s="19" t="inlineStr">
+        <is>
+          <t>EUR/kW</t>
+        </is>
+      </c>
+      <c r="E58" s="19" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (OCGT, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G58" s="19" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H58" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>Same cost file as PyPSA-Earth v0.10.0. For the new-build OCGT option (spec D1) and CO2 reporting (D9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="19" t="inlineStr">
+        <is>
+          <t>ocgt_fom</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>OCGT fixed O&amp;M</t>
+        </is>
+      </c>
+      <c r="C59" s="20" t="n">
+        <v>1.7795</v>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>%/year</t>
+        </is>
+      </c>
+      <c r="E59" s="19" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (OCGT, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G59" s="19" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Same cost file as PyPSA-Earth v0.10.0. For the new-build OCGT option (spec D1) and CO2 reporting (D9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="19" t="inlineStr">
+        <is>
+          <t>ocgt_lifetime</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>OCGT lifetime</t>
+        </is>
+      </c>
+      <c r="C60" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="D60" s="19" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E60" s="19" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (OCGT, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
+        </is>
+      </c>
+      <c r="G60" s="19" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H60" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>Same cost file as PyPSA-Earth v0.10.0. For the new-build OCGT option (spec D1) and CO2 reporting (D9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="19" t="inlineStr">
+        <is>
+          <t>gas_co2_intensity</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Natural gas CO2 intensity</t>
+        </is>
+      </c>
+      <c r="C61" s="20" t="n">
+        <v>0.198</v>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>tCO2/MWh_th</t>
+        </is>
+      </c>
+      <c r="E61" s="19" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, CO2 intensity); original: Stoichiometric calculation with 50 GJ/t CH4</t>
+        </is>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
+        </is>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Same cost file as PyPSA-Earth v0.10.0. For the new-build OCGT option (spec D1) and CO2 reporting (D9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="19" t="inlineStr">
+        <is>
+          <t>gas_for_power_2024_ktep_ncv</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Natural gas burnt for electricity 2024</t>
+        </is>
+      </c>
+      <c r="C62" s="20" t="n">
+        <v>3168</v>
+      </c>
+      <c r="D62" s="19" t="inlineStr">
+        <is>
+          <t>ktep (net CV)</t>
+        </is>
+      </c>
+      <c r="E62" s="19" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G62" s="19" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H62" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>Table of gas demand by use, 'Production d'électricité' 2024 = 3168 ktep-pci (PDF p.13). Cross-check of the fleet efficiency: 18,156 GWh / (3,168 x 11.63) GWh_th = 49.3%, vs 49.0% from specific consumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="19" t="inlineStr">
+        <is>
+          <t>cap_2024_selfgen_solar_lv_mw</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Self-generation solar, low voltage (rooftop), cumulative to 2024</t>
+        </is>
+      </c>
+      <c r="C63" s="20" t="n">
+        <v>315</v>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="E63" s="19" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G63" s="19" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H63" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>'Basse tension 315 MW' (PDF p.19). Not in the centralised fleet total of 6,012 MW.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="19" t="inlineStr">
+        <is>
+          <t>cap_2024_selfgen_solar_mvhv_mw</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Self-generation solar, medium/high voltage, authorised to 2024</t>
+        </is>
+      </c>
+      <c r="C64" s="20" t="n">
+        <v>125</v>
+      </c>
+      <c r="D64" s="19" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="E64" s="19" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
+        </is>
+      </c>
+      <c r="G64" s="19" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H64" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>'323 autorisations octroyées pour une puissance totale de 125 MW' (PDF p.19). Authorisations granted, not confirmed installations.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: link battery charger to discharger, add STEG reserve margin, two-way 3 h demand shift
</commit_message>
<xml_diff>
--- a/data/assumptions_register.xlsx
+++ b/data/assumptions_register.xlsx
@@ -71,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -95,6 +95,12 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -492,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -554,7 +560,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>re_target_2030</t>
         </is>
@@ -564,15 +570,15 @@
           <t>Renewable share of electricity generation, 2030</t>
         </is>
       </c>
-      <c r="C2" s="20" t="n">
+      <c r="C2" s="22" t="n">
         <v>0.35</v>
       </c>
-      <c r="D2" s="19" t="inlineStr">
+      <c r="D2" s="21" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E2" s="19" t="inlineStr">
+      <c r="E2" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -582,12 +588,12 @@
           <t>TAP, 9 Oct 2026: Head of Government reaffirms 35% target</t>
         </is>
       </c>
-      <c r="G2" s="19" t="inlineStr">
+      <c r="G2" s="21" t="inlineStr">
         <is>
           <t>https://www.tap.info.tn/fr/Portail-%C3%A0-la-Une-FR-top/20672933-%C3%A9nergie-la</t>
         </is>
       </c>
-      <c r="H2" s="19" t="inlineStr">
+      <c r="H2" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -599,7 +605,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>flex_cap_mw</t>
         </is>
@@ -609,15 +615,15 @@
           <t>Shiftable load cap (scenario S2-300)</t>
         </is>
       </c>
-      <c r="C3" s="20" t="n">
+      <c r="C3" s="22" t="n">
         <v>300</v>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="21" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
+      <c r="E3" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -627,12 +633,12 @@
           <t>TAP, 9 Oct 2026: action plan targets 300 MW peak-demand reduction</t>
         </is>
       </c>
-      <c r="G3" s="19" t="inlineStr">
+      <c r="G3" s="21" t="inlineStr">
         <is>
           <t>https://www.tap.info.tn/fr/Portail-%C3%A0-la-Une-FR-top/20672933-%C3%A9nergie-la</t>
         </is>
       </c>
-      <c r="H3" s="19" t="inlineStr">
+      <c r="H3" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -644,7 +650,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>flex_cap_hi_mw</t>
         </is>
@@ -654,22 +660,22 @@
           <t>Shiftable load cap, sensitivity (S2-600)</t>
         </is>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="22" t="n">
         <v>600</v>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="19" t="inlineStr"/>
-      <c r="H4" s="19" t="inlineStr">
+      <c r="G4" s="21" t="inlineStr"/>
+      <c r="H4" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -681,7 +687,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>flex_max_hours</t>
         </is>
@@ -691,22 +697,22 @@
           <t>Maximum shift duration</t>
         </is>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="19" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="E5" s="19" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="19" t="inlineStr"/>
-      <c r="H5" s="19" t="inlineStr">
+      <c r="G5" s="21" t="inlineStr"/>
+      <c r="H5" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -718,7 +724,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>gas_price_factor_lo</t>
         </is>
@@ -728,22 +734,22 @@
           <t>Gas price sensitivity, low</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>x base</t>
         </is>
       </c>
-      <c r="E6" s="19" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="19" t="inlineStr"/>
-      <c r="H6" s="19" t="inlineStr">
+      <c r="G6" s="21" t="inlineStr"/>
+      <c r="H6" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -755,7 +761,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>gas_price_factor_hi</t>
         </is>
@@ -765,22 +771,22 @@
           <t>Gas price sensitivity, high</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="22" t="n">
         <v>1.5</v>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>x base</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="19" t="inlineStr"/>
-      <c r="H7" s="19" t="inlineStr">
+      <c r="G7" s="21" t="inlineStr"/>
+      <c r="H7" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -792,7 +798,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>demand_growth</t>
         </is>
@@ -802,15 +808,15 @@
           <t>Electricity demand growth rate (STEG base case, applied 2024 -&gt; 2030)</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="22" t="n">
         <v>0.032</v>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>1/yr</t>
         </is>
       </c>
-      <c r="E8" s="19" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -820,12 +826,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.2-17 and p.5-34</t>
         </is>
       </c>
-      <c r="G8" s="19" t="inlineStr">
+      <c r="G8" s="21" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H8" s="19" t="inlineStr">
+      <c r="H8" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -837,7 +843,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>peak_ref_2030_mw</t>
         </is>
@@ -847,15 +853,15 @@
           <t>Reference 2030 peak demand</t>
         </is>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="22" t="n">
         <v>6000</v>
       </c>
-      <c r="D9" s="19" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E9" s="19" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -865,12 +871,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.2-17 and p.5-35</t>
         </is>
       </c>
-      <c r="G9" s="19" t="inlineStr">
+      <c r="G9" s="21" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H9" s="19" t="inlineStr">
+      <c r="H9" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -882,7 +888,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>discount_rate</t>
         </is>
@@ -892,15 +898,15 @@
           <t>Discount rate for annualising investment</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="22" t="n">
         <v>0.07099999999999999</v>
       </c>
-      <c r="D10" s="19" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>1/yr</t>
         </is>
       </c>
-      <c r="E10" s="19" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -910,12 +916,12 @@
           <t>PyPSA-Earth v0.10.0 config.default.yaml, costs.discountrate</t>
         </is>
       </c>
-      <c r="G10" s="19" t="inlineStr">
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>https://github.com/pypsa-meets-earth/pypsa-earth/blob/v0.10.0/config.default.yaml</t>
         </is>
       </c>
-      <c r="H10" s="19" t="inlineStr">
+      <c r="H10" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -927,7 +933,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>demand_2024_twh</t>
         </is>
@@ -937,15 +943,15 @@
           <t>Electricity demand 2024 (generation + net imports)</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="22" t="n">
         <v>22.507</v>
       </c>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E11" s="19" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -955,12 +961,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025), table 'ELECTRICITE', printed p.18</t>
         </is>
       </c>
-      <c r="G11" s="19" t="inlineStr">
+      <c r="G11" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H11" s="19" t="inlineStr">
+      <c r="H11" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -972,7 +978,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>imports_2024_twh</t>
         </is>
@@ -982,15 +988,15 @@
           <t>Net electricity imports 2024</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="22" t="n">
         <v>3.1131</v>
       </c>
-      <c r="D12" s="19" t="inlineStr">
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E12" s="19" t="inlineStr">
+      <c r="E12" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1000,12 +1006,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025), table 'ELECTRICITE', printed p.18</t>
         </is>
       </c>
-      <c r="G12" s="19" t="inlineStr">
+      <c r="G12" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H12" s="19" t="inlineStr">
+      <c r="H12" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -1017,7 +1023,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>gas_price_eur_per_mwh_th</t>
         </is>
@@ -1027,15 +1033,15 @@
           <t>Natural gas price (economic cost)</t>
         </is>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="22" t="n">
         <v>28.4158</v>
       </c>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="D13" s="21" t="inlineStr">
         <is>
           <t>EUR/MWh_th</t>
         </is>
       </c>
-      <c r="E13" s="19" t="inlineStr">
+      <c r="E13" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1045,12 +1051,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, fuel); original: World Bank Commodity Markets 2025 and ENTSO-E/ENTSOG TYNDP 2024</t>
         </is>
       </c>
-      <c r="G13" s="19" t="inlineStr">
+      <c r="G13" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H13" s="19" t="inlineStr">
+      <c r="H13" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -1062,7 +1068,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>toy_ccgt_investment</t>
         </is>
@@ -1072,15 +1078,15 @@
           <t>CCGT investment</t>
         </is>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="22" t="n">
         <v>1108.7166</v>
       </c>
-      <c r="D14" s="19" t="inlineStr">
+      <c r="D14" s="21" t="inlineStr">
         <is>
           <t>EUR/kW</t>
         </is>
       </c>
-      <c r="E14" s="19" t="inlineStr">
+      <c r="E14" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1090,12 +1096,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G14" s="19" t="inlineStr">
+      <c r="G14" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H14" s="19" t="inlineStr">
+      <c r="H14" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1107,7 +1113,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>toy_ccgt_fom</t>
         </is>
@@ -1117,15 +1123,15 @@
           <t>CCGT fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="22" t="n">
         <v>3.3494</v>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="D15" s="21" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E15" s="19" t="inlineStr">
+      <c r="E15" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1135,12 +1141,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G15" s="19" t="inlineStr">
+      <c r="G15" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H15" s="19" t="inlineStr">
+      <c r="H15" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1152,7 +1158,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>toy_ccgt_vom</t>
         </is>
@@ -1162,15 +1168,15 @@
           <t>CCGT variable O&amp;M</t>
         </is>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="22" t="n">
         <v>5.6104</v>
       </c>
-      <c r="D16" s="19" t="inlineStr">
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>EUR/MWh</t>
         </is>
       </c>
-      <c r="E16" s="19" t="inlineStr">
+      <c r="E16" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1180,12 +1186,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G16" s="19" t="inlineStr">
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H16" s="19" t="inlineStr">
+      <c r="H16" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1197,7 +1203,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>toy_ccgt_efficiency</t>
         </is>
@@ -1207,15 +1213,15 @@
           <t>CCGT electrical efficiency</t>
         </is>
       </c>
-      <c r="C17" s="20" t="n">
+      <c r="C17" s="22" t="n">
         <v>0.58</v>
       </c>
-      <c r="D17" s="19" t="inlineStr">
+      <c r="D17" s="21" t="inlineStr">
         <is>
           <t>per unit</t>
         </is>
       </c>
-      <c r="E17" s="19" t="inlineStr">
+      <c r="E17" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1225,12 +1231,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, efficiency); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G17" s="19" t="inlineStr">
+      <c r="G17" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H17" s="19" t="inlineStr">
+      <c r="H17" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1242,7 +1248,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>toy_ccgt_lifetime</t>
         </is>
@@ -1252,15 +1258,15 @@
           <t>CCGT lifetime</t>
         </is>
       </c>
-      <c r="C18" s="20" t="n">
+      <c r="C18" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D18" s="19" t="inlineStr">
+      <c r="D18" s="21" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E18" s="19" t="inlineStr">
+      <c r="E18" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1270,12 +1276,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G18" s="19" t="inlineStr">
+      <c r="G18" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H18" s="19" t="inlineStr">
+      <c r="H18" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1287,7 +1293,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>toy_solar_investment</t>
         </is>
@@ -1297,15 +1303,15 @@
           <t>Utility PV investment</t>
         </is>
       </c>
-      <c r="C19" s="20" t="n">
+      <c r="C19" s="22" t="n">
         <v>482.4785</v>
       </c>
-      <c r="D19" s="19" t="inlineStr">
+      <c r="D19" s="21" t="inlineStr">
         <is>
           <t>EUR/kW_e</t>
         </is>
       </c>
-      <c r="E19" s="19" t="inlineStr">
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1315,12 +1321,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G19" s="19" t="inlineStr">
+      <c r="G19" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H19" s="19" t="inlineStr">
+      <c r="H19" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1332,7 +1338,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>toy_solar_fom</t>
         </is>
@@ -1342,15 +1348,15 @@
           <t>Utility PV fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C20" s="20" t="n">
+      <c r="C20" s="22" t="n">
         <v>2.4757</v>
       </c>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="D20" s="21" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E20" s="19" t="inlineStr">
+      <c r="E20" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1360,12 +1366,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G20" s="19" t="inlineStr">
+      <c r="G20" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H20" s="19" t="inlineStr">
+      <c r="H20" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1377,7 +1383,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>toy_solar_lifetime</t>
         </is>
@@ -1387,15 +1393,15 @@
           <t>Utility PV lifetime</t>
         </is>
       </c>
-      <c r="C21" s="20" t="n">
+      <c r="C21" s="22" t="n">
         <v>40</v>
       </c>
-      <c r="D21" s="19" t="inlineStr">
+      <c r="D21" s="21" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E21" s="19" t="inlineStr">
+      <c r="E21" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1405,12 +1411,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (solar-utility, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G21" s="19" t="inlineStr">
+      <c r="G21" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H21" s="19" t="inlineStr">
+      <c r="H21" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1422,7 +1428,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="A22" s="21" t="inlineStr">
         <is>
           <t>toy_onwind_investment</t>
         </is>
@@ -1432,15 +1438,15 @@
           <t>Onshore wind investment</t>
         </is>
       </c>
-      <c r="C22" s="20" t="n">
+      <c r="C22" s="22" t="n">
         <v>1383.3059</v>
       </c>
-      <c r="D22" s="19" t="inlineStr">
+      <c r="D22" s="21" t="inlineStr">
         <is>
           <t>EUR/kW</t>
         </is>
       </c>
-      <c r="E22" s="19" t="inlineStr">
+      <c r="E22" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1450,12 +1456,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G22" s="19" t="inlineStr">
+      <c r="G22" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H22" s="19" t="inlineStr">
+      <c r="H22" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1467,7 +1473,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>toy_onwind_fom</t>
         </is>
@@ -1477,15 +1483,15 @@
           <t>Onshore wind fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C23" s="20" t="n">
+      <c r="C23" s="22" t="n">
         <v>1.2167</v>
       </c>
-      <c r="D23" s="19" t="inlineStr">
+      <c r="D23" s="21" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E23" s="19" t="inlineStr">
+      <c r="E23" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1495,12 +1501,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G23" s="19" t="inlineStr">
+      <c r="G23" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H23" s="19" t="inlineStr">
+      <c r="H23" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1512,7 +1518,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
+      <c r="A24" s="21" t="inlineStr">
         <is>
           <t>toy_onwind_vom</t>
         </is>
@@ -1522,15 +1528,15 @@
           <t>Onshore wind variable O&amp;M</t>
         </is>
       </c>
-      <c r="C24" s="20" t="n">
+      <c r="C24" s="22" t="n">
         <v>1.8033</v>
       </c>
-      <c r="D24" s="19" t="inlineStr">
+      <c r="D24" s="21" t="inlineStr">
         <is>
           <t>EUR/MWh</t>
         </is>
       </c>
-      <c r="E24" s="19" t="inlineStr">
+      <c r="E24" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1540,12 +1546,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G24" s="19" t="inlineStr">
+      <c r="G24" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H24" s="19" t="inlineStr">
+      <c r="H24" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1557,7 +1563,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>toy_onwind_lifetime</t>
         </is>
@@ -1567,15 +1573,15 @@
           <t>Onshore wind lifetime</t>
         </is>
       </c>
-      <c r="C25" s="20" t="n">
+      <c r="C25" s="22" t="n">
         <v>30</v>
       </c>
-      <c r="D25" s="19" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E25" s="19" t="inlineStr">
+      <c r="E25" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1585,12 +1591,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (onwind, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G25" s="19" t="inlineStr">
+      <c r="G25" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H25" s="19" t="inlineStr">
+      <c r="H25" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1602,7 +1608,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="A26" s="21" t="inlineStr">
         <is>
           <t>toy_battery_storage_investment</t>
         </is>
@@ -1612,15 +1618,15 @@
           <t>Battery energy (storage) investment</t>
         </is>
       </c>
-      <c r="C26" s="20" t="n">
+      <c r="C26" s="22" t="n">
         <v>189.861</v>
       </c>
-      <c r="D26" s="19" t="inlineStr">
+      <c r="D26" s="21" t="inlineStr">
         <is>
           <t>EUR/kWh</t>
         </is>
       </c>
-      <c r="E26" s="19" t="inlineStr">
+      <c r="E26" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1630,12 +1636,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery storage, investment); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G26" s="19" t="inlineStr">
+      <c r="G26" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H26" s="19" t="inlineStr">
+      <c r="H26" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1647,7 +1653,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>toy_battery_storage_lifetime</t>
         </is>
@@ -1657,15 +1663,15 @@
           <t>Battery energy (storage) lifetime</t>
         </is>
       </c>
-      <c r="C27" s="20" t="n">
+      <c r="C27" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D27" s="19" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E27" s="19" t="inlineStr">
+      <c r="E27" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1675,12 +1681,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery storage, lifetime); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G27" s="19" t="inlineStr">
+      <c r="G27" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H27" s="19" t="inlineStr">
+      <c r="H27" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1692,7 +1698,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="inlineStr">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>toy_battery_inverter_investment</t>
         </is>
@@ -1702,15 +1708,15 @@
           <t>Battery inverter (power) investment</t>
         </is>
       </c>
-      <c r="C28" s="20" t="n">
+      <c r="C28" s="22" t="n">
         <v>213.9279</v>
       </c>
-      <c r="D28" s="19" t="inlineStr">
+      <c r="D28" s="21" t="inlineStr">
         <is>
           <t>EUR/kW</t>
         </is>
       </c>
-      <c r="E28" s="19" t="inlineStr">
+      <c r="E28" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1720,12 +1726,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, investment); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G28" s="19" t="inlineStr">
+      <c r="G28" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H28" s="19" t="inlineStr">
+      <c r="H28" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1737,7 +1743,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>toy_battery_inverter_fom</t>
         </is>
@@ -1747,15 +1753,15 @@
           <t>Battery inverter fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C29" s="20" t="n">
+      <c r="C29" s="22" t="n">
         <v>0.3375</v>
       </c>
-      <c r="D29" s="19" t="inlineStr">
+      <c r="D29" s="21" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E29" s="19" t="inlineStr">
+      <c r="E29" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1765,12 +1771,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, FOM); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G29" s="19" t="inlineStr">
+      <c r="G29" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H29" s="19" t="inlineStr">
+      <c r="H29" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1782,7 +1788,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="inlineStr">
+      <c r="A30" s="21" t="inlineStr">
         <is>
           <t>toy_battery_inverter_efficiency</t>
         </is>
@@ -1792,15 +1798,15 @@
           <t>Battery round-trip efficiency (source: 'Round trip efficiency DC')</t>
         </is>
       </c>
-      <c r="C30" s="20" t="n">
+      <c r="C30" s="22" t="n">
         <v>0.96</v>
       </c>
-      <c r="D30" s="19" t="inlineStr">
+      <c r="D30" s="21" t="inlineStr">
         <is>
           <t>per unit</t>
         </is>
       </c>
-      <c r="E30" s="19" t="inlineStr">
+      <c r="E30" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1810,12 +1816,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, efficiency); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx</t>
         </is>
       </c>
-      <c r="G30" s="19" t="inlineStr">
+      <c r="G30" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H30" s="19" t="inlineStr">
+      <c r="H30" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1827,7 +1833,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="A31" s="21" t="inlineStr">
         <is>
           <t>toy_battery_inverter_lifetime</t>
         </is>
@@ -1837,15 +1843,15 @@
           <t>Battery inverter lifetime</t>
         </is>
       </c>
-      <c r="C31" s="20" t="n">
+      <c r="C31" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="D31" s="19" t="inlineStr">
+      <c r="D31" s="21" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E31" s="19" t="inlineStr">
+      <c r="E31" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1855,12 +1861,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (battery inverter, lifetime); original: Danish Energy Agency, inputs/technology_data_catalogue_for_energy_storage.xlsx, Note K.</t>
         </is>
       </c>
-      <c r="G31" s="19" t="inlineStr">
+      <c r="G31" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H31" s="19" t="inlineStr">
+      <c r="H31" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1872,7 +1878,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="A32" s="21" t="inlineStr">
         <is>
           <t>toy_gas_fuel</t>
         </is>
@@ -1882,15 +1888,15 @@
           <t>Natural gas fuel cost</t>
         </is>
       </c>
-      <c r="C32" s="20" t="n">
+      <c r="C32" s="22" t="n">
         <v>28.4158</v>
       </c>
-      <c r="D32" s="19" t="inlineStr">
+      <c r="D32" s="21" t="inlineStr">
         <is>
           <t>EUR/MWh_th</t>
         </is>
       </c>
-      <c r="E32" s="19" t="inlineStr">
+      <c r="E32" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1900,12 +1906,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, fuel); original: World Bank (2025) Commodity Markets, https://www.worldbank.org/en/research/commodity-markets; and ENTSO-E &amp; ENTSOG TYNDP 2024 Scenarios Inputs Commodity Prices, https://2024-data.entsos-tyndp-scenarios.eu/files/scenarios-inputs/Prices.zip, accessed: 2026-02-03.</t>
         </is>
       </c>
-      <c r="G32" s="19" t="inlineStr">
+      <c r="G32" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H32" s="19" t="inlineStr">
+      <c r="H32" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1917,7 +1923,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="A33" s="21" t="inlineStr">
         <is>
           <t>toy_gas_co2_intensity</t>
         </is>
@@ -1927,15 +1933,15 @@
           <t>Natural gas CO2 intensity</t>
         </is>
       </c>
-      <c r="C33" s="20" t="n">
+      <c r="C33" s="22" t="n">
         <v>0.198</v>
       </c>
-      <c r="D33" s="19" t="inlineStr">
+      <c r="D33" s="21" t="inlineStr">
         <is>
           <t>tCO2/MWh_th</t>
         </is>
       </c>
-      <c r="E33" s="19" t="inlineStr">
+      <c r="E33" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -1945,12 +1951,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, CO2 intensity); original: Stoichiometric calculation with 50 GJ/t CH4</t>
         </is>
       </c>
-      <c r="G33" s="19" t="inlineStr">
+      <c r="G33" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H33" s="19" t="inlineStr">
+      <c r="H33" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1962,7 +1968,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="19" t="inlineStr">
+      <c r="A34" s="21" t="inlineStr">
         <is>
           <t>toy_battery_max_hours</t>
         </is>
@@ -1972,22 +1978,22 @@
           <t>Toy battery energy-to-power ratio</t>
         </is>
       </c>
-      <c r="C34" s="20" t="n">
+      <c r="C34" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="D34" s="19" t="inlineStr">
+      <c r="D34" s="21" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="E34" s="19" t="inlineStr">
+      <c r="E34" s="21" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr"/>
-      <c r="G34" s="19" t="inlineStr"/>
-      <c r="H34" s="19" t="inlineStr">
+      <c r="G34" s="21" t="inlineStr"/>
+      <c r="H34" s="21" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
@@ -1999,7 +2005,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="19" t="inlineStr">
+      <c r="A35" s="21" t="inlineStr">
         <is>
           <t>cap_2024_ccgt_mw</t>
         </is>
@@ -2009,15 +2015,15 @@
           <t>Net installed capacity 2024: combined cycle</t>
         </is>
       </c>
-      <c r="C35" s="20" t="n">
+      <c r="C35" s="22" t="n">
         <v>2527</v>
       </c>
-      <c r="D35" s="19" t="inlineStr">
+      <c r="D35" s="21" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E35" s="19" t="inlineStr">
+      <c r="E35" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2027,12 +2033,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G35" s="19" t="inlineStr">
+      <c r="G35" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H35" s="19" t="inlineStr">
+      <c r="H35" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2044,7 +2050,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="19" t="inlineStr">
+      <c r="A36" s="21" t="inlineStr">
         <is>
           <t>cap_2024_ocgt_mw</t>
         </is>
@@ -2054,15 +2060,15 @@
           <t>Net installed capacity 2024: gas turbines (open cycle)</t>
         </is>
       </c>
-      <c r="C36" s="20" t="n">
+      <c r="C36" s="22" t="n">
         <v>2457</v>
       </c>
-      <c r="D36" s="19" t="inlineStr">
+      <c r="D36" s="21" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E36" s="19" t="inlineStr">
+      <c r="E36" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2072,12 +2078,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G36" s="19" t="inlineStr">
+      <c r="G36" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H36" s="19" t="inlineStr">
+      <c r="H36" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2089,7 +2095,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="19" t="inlineStr">
+      <c r="A37" s="21" t="inlineStr">
         <is>
           <t>cap_2024_steam_mw</t>
         </is>
@@ -2099,15 +2105,15 @@
           <t>Net installed capacity 2024: steam turbines</t>
         </is>
       </c>
-      <c r="C37" s="20" t="n">
+      <c r="C37" s="22" t="n">
         <v>660</v>
       </c>
-      <c r="D37" s="19" t="inlineStr">
+      <c r="D37" s="21" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E37" s="19" t="inlineStr">
+      <c r="E37" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2117,12 +2123,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G37" s="19" t="inlineStr">
+      <c r="G37" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H37" s="19" t="inlineStr">
+      <c r="H37" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2134,7 +2140,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="19" t="inlineStr">
+      <c r="A38" s="21" t="inlineStr">
         <is>
           <t>cap_2024_re_mw</t>
         </is>
@@ -2144,15 +2150,15 @@
           <t>Net installed capacity 2024: renewables (hydro + wind + solar, centralised)</t>
         </is>
       </c>
-      <c r="C38" s="20" t="n">
+      <c r="C38" s="22" t="n">
         <v>368</v>
       </c>
-      <c r="D38" s="19" t="inlineStr">
+      <c r="D38" s="21" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E38" s="19" t="inlineStr">
+      <c r="E38" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2162,12 +2168,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G38" s="19" t="inlineStr">
+      <c r="G38" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H38" s="19" t="inlineStr">
+      <c r="H38" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2179,7 +2185,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="19" t="inlineStr">
+      <c r="A39" s="21" t="inlineStr">
         <is>
           <t>cap_2024_total_mw</t>
         </is>
@@ -2189,15 +2195,15 @@
           <t>Net installed capacity 2024: total</t>
         </is>
       </c>
-      <c r="C39" s="20" t="n">
+      <c r="C39" s="22" t="n">
         <v>6012</v>
       </c>
-      <c r="D39" s="19" t="inlineStr">
+      <c r="D39" s="21" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E39" s="19" t="inlineStr">
+      <c r="E39" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2207,12 +2213,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G39" s="19" t="inlineStr">
+      <c r="G39" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H39" s="19" t="inlineStr">
+      <c r="H39" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2224,7 +2230,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="19" t="inlineStr">
+      <c r="A40" s="21" t="inlineStr">
         <is>
           <t>gen_2024_gas_twh</t>
         </is>
@@ -2234,15 +2240,15 @@
           <t>Electricity generation 2024: natural gas</t>
         </is>
       </c>
-      <c r="C40" s="20" t="n">
+      <c r="C40" s="22" t="n">
         <v>18.156</v>
       </c>
-      <c r="D40" s="19" t="inlineStr">
+      <c r="D40" s="21" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E40" s="19" t="inlineStr">
+      <c r="E40" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2252,12 +2258,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G40" s="19" t="inlineStr">
+      <c r="G40" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H40" s="19" t="inlineStr">
+      <c r="H40" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2269,7 +2275,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="19" t="inlineStr">
+      <c r="A41" s="21" t="inlineStr">
         <is>
           <t>gen_2024_oil_twh</t>
         </is>
@@ -2279,15 +2285,15 @@
           <t>Electricity generation 2024: fuel oil + gasoil</t>
         </is>
       </c>
-      <c r="C41" s="20" t="n">
+      <c r="C41" s="22" t="n">
         <v>0.07190000000000001</v>
       </c>
-      <c r="D41" s="19" t="inlineStr">
+      <c r="D41" s="21" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E41" s="19" t="inlineStr">
+      <c r="E41" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2297,12 +2303,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G41" s="19" t="inlineStr">
+      <c r="G41" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H41" s="19" t="inlineStr">
+      <c r="H41" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2314,7 +2320,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="19" t="inlineStr">
+      <c r="A42" s="21" t="inlineStr">
         <is>
           <t>gen_2024_hydro_twh</t>
         </is>
@@ -2324,15 +2330,15 @@
           <t>Electricity generation 2024: hydro</t>
         </is>
       </c>
-      <c r="C42" s="20" t="n">
+      <c r="C42" s="22" t="n">
         <v>0.016</v>
       </c>
-      <c r="D42" s="19" t="inlineStr">
+      <c r="D42" s="21" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E42" s="19" t="inlineStr">
+      <c r="E42" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2342,12 +2348,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G42" s="19" t="inlineStr">
+      <c r="G42" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H42" s="19" t="inlineStr">
+      <c r="H42" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2359,7 +2365,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="19" t="inlineStr">
+      <c r="A43" s="21" t="inlineStr">
         <is>
           <t>gen_2024_wind_twh</t>
         </is>
@@ -2369,15 +2375,15 @@
           <t>Electricity generation 2024: wind</t>
         </is>
       </c>
-      <c r="C43" s="20" t="n">
+      <c r="C43" s="22" t="n">
         <v>0.337</v>
       </c>
-      <c r="D43" s="19" t="inlineStr">
+      <c r="D43" s="21" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E43" s="19" t="inlineStr">
+      <c r="E43" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2387,12 +2393,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G43" s="19" t="inlineStr">
+      <c r="G43" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H43" s="19" t="inlineStr">
+      <c r="H43" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2404,7 +2410,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="19" t="inlineStr">
+      <c r="A44" s="21" t="inlineStr">
         <is>
           <t>gen_2024_solar_twh</t>
         </is>
@@ -2414,15 +2420,15 @@
           <t>Electricity generation 2024: solar PV (STEG + IPP + self-generation)</t>
         </is>
       </c>
-      <c r="C44" s="20" t="n">
+      <c r="C44" s="22" t="n">
         <v>0.6278</v>
       </c>
-      <c r="D44" s="19" t="inlineStr">
+      <c r="D44" s="21" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E44" s="19" t="inlineStr">
+      <c r="E44" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2432,12 +2438,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G44" s="19" t="inlineStr">
+      <c r="G44" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H44" s="19" t="inlineStr">
+      <c r="H44" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2449,7 +2455,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="19" t="inlineStr">
+      <c r="A45" s="21" t="inlineStr">
         <is>
           <t>gen_2024_total_twh</t>
         </is>
@@ -2459,15 +2465,15 @@
           <t>Electricity generation 2024: total</t>
         </is>
       </c>
-      <c r="C45" s="20" t="n">
+      <c r="C45" s="22" t="n">
         <v>19.208</v>
       </c>
-      <c r="D45" s="19" t="inlineStr">
+      <c r="D45" s="21" t="inlineStr">
         <is>
           <t>TWh</t>
         </is>
       </c>
-      <c r="E45" s="19" t="inlineStr">
+      <c r="E45" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2477,12 +2483,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G45" s="19" t="inlineStr">
+      <c r="G45" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H45" s="19" t="inlineStr">
+      <c r="H45" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2494,7 +2500,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="19" t="inlineStr">
+      <c r="A46" s="21" t="inlineStr">
         <is>
           <t>gas_share_2024</t>
         </is>
@@ -2504,15 +2510,15 @@
           <t>Gas share of electricity generation 2024</t>
         </is>
       </c>
-      <c r="C46" s="20" t="n">
+      <c r="C46" s="22" t="n">
         <v>0.945</v>
       </c>
-      <c r="D46" s="19" t="inlineStr">
+      <c r="D46" s="21" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E46" s="19" t="inlineStr">
+      <c r="E46" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2522,12 +2528,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G46" s="19" t="inlineStr">
+      <c r="G46" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H46" s="19" t="inlineStr">
+      <c r="H46" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2539,7 +2545,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="19" t="inlineStr">
+      <c r="A47" s="21" t="inlineStr">
         <is>
           <t>peak_2024_mw</t>
         </is>
@@ -2549,15 +2555,15 @@
           <t>Peak electricity demand 2024</t>
         </is>
       </c>
-      <c r="C47" s="20" t="n">
+      <c r="C47" s="22" t="n">
         <v>4888</v>
       </c>
-      <c r="D47" s="19" t="inlineStr">
+      <c r="D47" s="21" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E47" s="19" t="inlineStr">
+      <c r="E47" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2567,12 +2573,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G47" s="19" t="inlineStr">
+      <c r="G47" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H47" s="19" t="inlineStr">
+      <c r="H47" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2584,7 +2590,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="19" t="inlineStr">
+      <c r="A48" s="21" t="inlineStr">
         <is>
           <t>steg_specific_consumption_2024</t>
         </is>
@@ -2594,15 +2600,15 @@
           <t>STEG fleet specific fuel consumption 2024</t>
         </is>
       </c>
-      <c r="C48" s="20" t="n">
+      <c r="C48" s="22" t="n">
         <v>194.8</v>
       </c>
-      <c r="D48" s="19" t="inlineStr">
+      <c r="D48" s="21" t="inlineStr">
         <is>
           <t>toe(GCV)/GWh</t>
         </is>
       </c>
-      <c r="E48" s="19" t="inlineStr">
+      <c r="E48" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2612,12 +2618,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G48" s="19" t="inlineStr">
+      <c r="G48" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H48" s="19" t="inlineStr">
+      <c r="H48" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2629,7 +2635,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="19" t="inlineStr">
+      <c r="A49" s="21" t="inlineStr">
         <is>
           <t>steg_demand_2030_gwh</t>
         </is>
@@ -2639,15 +2645,15 @@
           <t>STEG forecast of 2030 electricity demand</t>
         </is>
       </c>
-      <c r="C49" s="20" t="n">
+      <c r="C49" s="22" t="n">
         <v>28362</v>
       </c>
-      <c r="D49" s="19" t="inlineStr">
+      <c r="D49" s="21" t="inlineStr">
         <is>
           <t>GWh</t>
         </is>
       </c>
-      <c r="E49" s="19" t="inlineStr">
+      <c r="E49" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2657,12 +2663,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.2-17</t>
         </is>
       </c>
-      <c r="G49" s="19" t="inlineStr">
+      <c r="G49" s="21" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H49" s="19" t="inlineStr">
+      <c r="H49" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2674,7 +2680,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="19" t="inlineStr">
+      <c r="A50" s="21" t="inlineStr">
         <is>
           <t>load_factor_2030</t>
         </is>
@@ -2684,15 +2690,15 @@
           <t>STEG 2030 forecast: annual load factor</t>
         </is>
       </c>
-      <c r="C50" s="20" t="n">
+      <c r="C50" s="22" t="n">
         <v>0.54</v>
       </c>
-      <c r="D50" s="19" t="inlineStr">
+      <c r="D50" s="21" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E50" s="19" t="inlineStr">
+      <c r="E50" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2702,12 +2708,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.5-34</t>
         </is>
       </c>
-      <c r="G50" s="19" t="inlineStr">
+      <c r="G50" s="21" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H50" s="19" t="inlineStr">
+      <c r="H50" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2719,7 +2725,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="19" t="inlineStr">
+      <c r="A51" s="21" t="inlineStr">
         <is>
           <t>min_to_peak_2030</t>
         </is>
@@ -2729,15 +2735,15 @@
           <t>STEG 2030 forecast: minimum-to-peak load ratio</t>
         </is>
       </c>
-      <c r="C51" s="20" t="n">
+      <c r="C51" s="22" t="n">
         <v>0.34</v>
       </c>
-      <c r="D51" s="19" t="inlineStr">
+      <c r="D51" s="21" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="E51" s="19" t="inlineStr">
+      <c r="E51" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2747,12 +2753,12 @@
           <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), quoting STEG's base-case forecast, p.5-35</t>
         </is>
       </c>
-      <c r="G51" s="19" t="inlineStr">
+      <c r="G51" s="21" t="inlineStr">
         <is>
           <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
         </is>
       </c>
-      <c r="H51" s="19" t="inlineStr">
+      <c r="H51" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2764,7 +2770,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="19" t="inlineStr">
+      <c r="A52" s="21" t="inlineStr">
         <is>
           <t>ccgt_efficiency</t>
         </is>
@@ -2774,15 +2780,15 @@
           <t>CCGT electrical efficiency (new build)</t>
         </is>
       </c>
-      <c r="C52" s="20" t="n">
+      <c r="C52" s="22" t="n">
         <v>0.58</v>
       </c>
-      <c r="D52" s="19" t="inlineStr">
+      <c r="D52" s="21" t="inlineStr">
         <is>
           <t>per unit</t>
         </is>
       </c>
-      <c r="E52" s="19" t="inlineStr">
+      <c r="E52" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2792,12 +2798,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, efficiency); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G52" s="19" t="inlineStr">
+      <c r="G52" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H52" s="19" t="inlineStr">
+      <c r="H52" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2809,7 +2815,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="19" t="inlineStr">
+      <c r="A53" s="21" t="inlineStr">
         <is>
           <t>ccgt_vom</t>
         </is>
@@ -2819,15 +2825,15 @@
           <t>CCGT variable O&amp;M</t>
         </is>
       </c>
-      <c r="C53" s="20" t="n">
+      <c r="C53" s="22" t="n">
         <v>5.6104</v>
       </c>
-      <c r="D53" s="19" t="inlineStr">
+      <c r="D53" s="21" t="inlineStr">
         <is>
           <t>EUR/MWh</t>
         </is>
       </c>
-      <c r="E53" s="19" t="inlineStr">
+      <c r="E53" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2837,12 +2843,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (CCGT, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G53" s="19" t="inlineStr">
+      <c r="G53" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H53" s="19" t="inlineStr">
+      <c r="H53" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2854,7 +2860,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="19" t="inlineStr">
+      <c r="A54" s="21" t="inlineStr">
         <is>
           <t>ocgt_efficiency</t>
         </is>
@@ -2864,15 +2870,15 @@
           <t>OCGT electrical efficiency (new build)</t>
         </is>
       </c>
-      <c r="C54" s="20" t="n">
+      <c r="C54" s="22" t="n">
         <v>0.41</v>
       </c>
-      <c r="D54" s="19" t="inlineStr">
+      <c r="D54" s="21" t="inlineStr">
         <is>
           <t>per unit</t>
         </is>
       </c>
-      <c r="E54" s="19" t="inlineStr">
+      <c r="E54" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2882,12 +2888,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (OCGT, efficiency); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G54" s="19" t="inlineStr">
+      <c r="G54" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H54" s="19" t="inlineStr">
+      <c r="H54" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2899,7 +2905,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="19" t="inlineStr">
+      <c r="A55" s="21" t="inlineStr">
         <is>
           <t>ocgt_vom</t>
         </is>
@@ -2909,15 +2915,15 @@
           <t>OCGT variable O&amp;M</t>
         </is>
       </c>
-      <c r="C55" s="20" t="n">
+      <c r="C55" s="22" t="n">
         <v>6.0111</v>
       </c>
-      <c r="D55" s="19" t="inlineStr">
+      <c r="D55" s="21" t="inlineStr">
         <is>
           <t>EUR/MWh</t>
         </is>
       </c>
-      <c r="E55" s="19" t="inlineStr">
+      <c r="E55" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2927,12 +2933,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (OCGT, VOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G55" s="19" t="inlineStr">
+      <c r="G55" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H55" s="19" t="inlineStr">
+      <c r="H55" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2944,7 +2950,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="19" t="inlineStr">
+      <c r="A56" s="21" t="inlineStr">
         <is>
           <t>gas_ncv_per_gcv</t>
         </is>
@@ -2954,15 +2960,15 @@
           <t>Natural gas: net / gross calorific value</t>
         </is>
       </c>
-      <c r="C56" s="20" t="n">
+      <c r="C56" s="22" t="n">
         <v>0.9</v>
       </c>
-      <c r="D56" s="19" t="inlineStr">
+      <c r="D56" s="21" t="inlineStr">
         <is>
           <t>ratio</t>
         </is>
       </c>
-      <c r="E56" s="19" t="inlineStr">
+      <c r="E56" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -2972,12 +2978,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024, conversion table (PDF p.22)</t>
         </is>
       </c>
-      <c r="G56" s="19" t="inlineStr">
+      <c r="G56" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H56" s="19" t="inlineStr">
+      <c r="H56" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -2989,7 +2995,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="19" t="inlineStr">
+      <c r="A57" s="21" t="inlineStr">
         <is>
           <t>existing_gas_efficiency_factor</t>
         </is>
@@ -2999,15 +3005,15 @@
           <t>Efficiency factor for existing gas units (calibrated)</t>
         </is>
       </c>
-      <c r="C57" s="20" t="n">
+      <c r="C57" s="22" t="n">
         <v>0.8633999999999999</v>
       </c>
-      <c r="D57" s="19" t="inlineStr">
+      <c r="D57" s="21" t="inlineStr">
         <is>
           <t>x tech-data</t>
         </is>
       </c>
-      <c r="E57" s="19" t="inlineStr">
+      <c r="E57" s="21" t="inlineStr">
         <is>
           <t>assumption</t>
         </is>
@@ -3017,12 +3023,12 @@
           <t>Calibrated (Task 10) so the dispatch-only 2024 run matches STEG's measured fuel use: ONEM Memento 2024, specific consumption 194.8 toe(PCS)/GWh, PCI = 0.9 PCS</t>
         </is>
       </c>
-      <c r="G57" s="19" t="inlineStr">
+      <c r="G57" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H57" s="19" t="inlineStr">
+      <c r="H57" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -3034,7 +3040,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="19" t="inlineStr">
+      <c r="A58" s="21" t="inlineStr">
         <is>
           <t>ocgt_investment</t>
         </is>
@@ -3044,15 +3050,15 @@
           <t>OCGT investment (new build)</t>
         </is>
       </c>
-      <c r="C58" s="20" t="n">
+      <c r="C58" s="22" t="n">
         <v>581.3949</v>
       </c>
-      <c r="D58" s="19" t="inlineStr">
+      <c r="D58" s="21" t="inlineStr">
         <is>
           <t>EUR/kW</t>
         </is>
       </c>
-      <c r="E58" s="19" t="inlineStr">
+      <c r="E58" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -3062,12 +3068,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (OCGT, investment); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G58" s="19" t="inlineStr">
+      <c r="G58" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H58" s="19" t="inlineStr">
+      <c r="H58" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -3079,7 +3085,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="19" t="inlineStr">
+      <c r="A59" s="21" t="inlineStr">
         <is>
           <t>ocgt_fom</t>
         </is>
@@ -3089,15 +3095,15 @@
           <t>OCGT fixed O&amp;M</t>
         </is>
       </c>
-      <c r="C59" s="20" t="n">
+      <c r="C59" s="22" t="n">
         <v>1.7795</v>
       </c>
-      <c r="D59" s="19" t="inlineStr">
+      <c r="D59" s="21" t="inlineStr">
         <is>
           <t>%/year</t>
         </is>
       </c>
-      <c r="E59" s="19" t="inlineStr">
+      <c r="E59" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -3107,12 +3113,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (OCGT, FOM); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G59" s="19" t="inlineStr">
+      <c r="G59" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H59" s="19" t="inlineStr">
+      <c r="H59" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -3124,7 +3130,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="19" t="inlineStr">
+      <c r="A60" s="21" t="inlineStr">
         <is>
           <t>ocgt_lifetime</t>
         </is>
@@ -3134,15 +3140,15 @@
           <t>OCGT lifetime</t>
         </is>
       </c>
-      <c r="C60" s="20" t="n">
+      <c r="C60" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D60" s="19" t="inlineStr">
+      <c r="D60" s="21" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E60" s="19" t="inlineStr">
+      <c r="E60" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -3152,12 +3158,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (OCGT, lifetime); original: Danish Energy Agency, inputs/technology_data_for_el_and_dh.xlsx</t>
         </is>
       </c>
-      <c r="G60" s="19" t="inlineStr">
+      <c r="G60" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H60" s="19" t="inlineStr">
+      <c r="H60" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -3169,7 +3175,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="19" t="inlineStr">
+      <c r="A61" s="21" t="inlineStr">
         <is>
           <t>gas_co2_intensity</t>
         </is>
@@ -3179,15 +3185,15 @@
           <t>Natural gas CO2 intensity</t>
         </is>
       </c>
-      <c r="C61" s="20" t="n">
+      <c r="C61" s="22" t="n">
         <v>0.198</v>
       </c>
-      <c r="D61" s="19" t="inlineStr">
+      <c r="D61" s="21" t="inlineStr">
         <is>
           <t>tCO2/MWh_th</t>
         </is>
       </c>
-      <c r="E61" s="19" t="inlineStr">
+      <c r="E61" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -3197,12 +3203,12 @@
           <t>PyPSA technology-data v0.15.0 costs_2030.csv (gas, CO2 intensity); original: Stoichiometric calculation with 50 GJ/t CH4</t>
         </is>
       </c>
-      <c r="G61" s="19" t="inlineStr">
+      <c r="G61" s="21" t="inlineStr">
         <is>
           <t>https://github.com/PyPSA/technology-data/blob/v0.15.0/outputs/costs_2030.csv</t>
         </is>
       </c>
-      <c r="H61" s="19" t="inlineStr">
+      <c r="H61" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -3214,7 +3220,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="19" t="inlineStr">
+      <c r="A62" s="21" t="inlineStr">
         <is>
           <t>gas_for_power_2024_ktep_ncv</t>
         </is>
@@ -3224,15 +3230,15 @@
           <t>Natural gas burnt for electricity 2024</t>
         </is>
       </c>
-      <c r="C62" s="20" t="n">
+      <c r="C62" s="22" t="n">
         <v>3168</v>
       </c>
-      <c r="D62" s="19" t="inlineStr">
+      <c r="D62" s="21" t="inlineStr">
         <is>
           <t>ktep (net CV)</t>
         </is>
       </c>
-      <c r="E62" s="19" t="inlineStr">
+      <c r="E62" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -3242,12 +3248,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G62" s="19" t="inlineStr">
+      <c r="G62" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H62" s="19" t="inlineStr">
+      <c r="H62" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -3259,7 +3265,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="19" t="inlineStr">
+      <c r="A63" s="21" t="inlineStr">
         <is>
           <t>cap_2024_selfgen_solar_lv_mw</t>
         </is>
@@ -3269,15 +3275,15 @@
           <t>Self-generation solar, low voltage (rooftop), cumulative to 2024</t>
         </is>
       </c>
-      <c r="C63" s="20" t="n">
+      <c r="C63" s="22" t="n">
         <v>315</v>
       </c>
-      <c r="D63" s="19" t="inlineStr">
+      <c r="D63" s="21" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E63" s="19" t="inlineStr">
+      <c r="E63" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -3287,12 +3293,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G63" s="19" t="inlineStr">
+      <c r="G63" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H63" s="19" t="inlineStr">
+      <c r="H63" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -3304,7 +3310,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="19" t="inlineStr">
+      <c r="A64" s="21" t="inlineStr">
         <is>
           <t>cap_2024_selfgen_solar_mvhv_mw</t>
         </is>
@@ -3314,15 +3320,15 @@
           <t>Self-generation solar, medium/high voltage, authorised to 2024</t>
         </is>
       </c>
-      <c r="C64" s="20" t="n">
+      <c r="C64" s="22" t="n">
         <v>125</v>
       </c>
-      <c r="D64" s="19" t="inlineStr">
+      <c r="D64" s="21" t="inlineStr">
         <is>
           <t>MW</t>
         </is>
       </c>
-      <c r="E64" s="19" t="inlineStr">
+      <c r="E64" s="21" t="inlineStr">
         <is>
           <t>sourced</t>
         </is>
@@ -3332,12 +3338,12 @@
           <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025)</t>
         </is>
       </c>
-      <c r="G64" s="19" t="inlineStr">
+      <c r="G64" s="21" t="inlineStr">
         <is>
           <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
         </is>
       </c>
-      <c r="H64" s="19" t="inlineStr">
+      <c r="H64" s="21" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
@@ -3345,6 +3351,51 @@
       <c r="I64" s="3" t="inlineStr">
         <is>
           <t>'323 autorisations octroyées pour une puissance totale de 125 MW' (PDF p.19). Authorisations granted, not confirmed installations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="21" t="inlineStr">
+        <is>
+          <t>reserve_margin</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Planning reserve margin on firm capacity (lower bound of STEG target)</t>
+        </is>
+      </c>
+      <c r="C65" s="22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D65" s="21" t="inlineStr">
+        <is>
+          <t>share of peak</t>
+        </is>
+      </c>
+      <c r="E65" s="21" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), p.5-33</t>
+        </is>
+      </c>
+      <c r="G65" s="21" t="inlineStr">
+        <is>
+          <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
+        </is>
+      </c>
+      <c r="H65" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>STEG supply reliability target: 'Reserve Margin: 10-15% of yearly power peak'. Lower bound used (author, 2026-10-28). Firm = gas + hydro; wind, solar, batteries and shifted load get no firm credit.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: add sourced context on Tunisia's gas supply and power sector
Nine rows, all from the ONEM Memento 2024 and the JICA 2022 survey already used by the study; marked as context, not used by the model.
</commit_message>
<xml_diff>
--- a/data/assumptions_register.xlsx
+++ b/data/assumptions_register.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3396,6 +3396,411 @@
       <c r="I65" s="3" t="inlineStr">
         <is>
           <t>STEG supply reliability target: 'Reserve Margin: 10-15% of yearly power peak'. Lower bound used (author, 2026-10-28). Firm = gas + hydro; wind, solar, batteries and shifted load get no firm credit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>gas_supply_domestic_2024_ktep</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Natural gas supply 2024: national production</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>1212</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>ktep (net CV)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025), table 'Gaz naturel' (approvisionnement, ktep-pci)</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Context for the learning guide; not used by the model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>gas_supply_royalty_2024_ktep</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Natural gas supply 2024: royalty on Algerian gas crossing Tunisia (redevance)</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>909</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>ktep (net CV)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025), table 'Gaz naturel' (approvisionnement, ktep-pci)</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Context for the learning guide; not used by the model. Tunisia is the transit country for the Algeria-Italy gas pipeline (JICA 2022, p.2-2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>gas_supply_purchases_2024_ktep</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Natural gas supply 2024: purchases of Algerian gas</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>2290</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>ktep (net CV)</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025), table 'Gaz naturel' (approvisionnement, ktep-pci)</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Context for the learning guide; not used by the model. ONEM: purchases fell 4% because more electricity was bought directly, mainly from Algeria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>energy_independence_2024</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Energy independence rate 2024 (national primary resources / primary demand)</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025), 'Bilan d'énergie primaire'</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Context for the learning guide; not used by the model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>steg_established_year</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Year STEG (state-owned electricity and gas company) was established</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>1962</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), p.2-1</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Context for the learning guide; not used by the model. STEG is vertically integrated: transmission, distribution and gas supply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>steg_generation_share</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>STEG's share of total power generation</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), p.2-1</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Context for the learning guide; not used by the model. Independent producers make the remaining ~14% (generation opened in 1996).</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>anme_established_year</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Year ANME (national energy efficiency agency) was established</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>1985</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), p.2-1</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Context for the learning guide; not used by the model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>tsp_re_target_2030</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Renewable share target 2030 in the Tunisian Solar Plan (ANME, 2012)</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), p.2-2</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Context for the learning guide; not used by the model. Later raised to 35% (see re_target_2030).</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>indc_co2_intensity_cut_2030</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>INDC goal: cut in CO2 emission intensity by 2030 vs 2010</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>JICA / TEPSCO / KPMG, Data Collection Survey on Power Sector in Tunisia, Final Report (Mar 2022), p.2-2</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://openjicareport.jica.go.jp/pdf/12342283.pdf</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Context for the learning guide; not used by the model. Submitted to the UNFCCC in September 2015.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add the learning path
Seven short chapters and a glossary, from Tunisia's gas-fired power system to running your own scenario. The chapter 7 exercise (a 12% saving) was run on the real network and its output is quoted as printed. Adds the 2023 gas production row used in chapter 1.
</commit_message>
<xml_diff>
--- a/data/assumptions_register.xlsx
+++ b/data/assumptions_register.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3801,6 +3801,51 @@
       <c r="I74" t="inlineStr">
         <is>
           <t>Context for the learning guide; not used by the model. Submitted to the UNFCCC in September 2015.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>gas_supply_domestic_2023_ktep</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Natural gas supply 2023: national production</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>1607</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>ktep (net CV)</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>ONEM / Ministry of Industry, Mines and Energy, Memento du secteur de l'énergie, Chiffres de 2024 (Aug 2025), table 'Gaz naturel' (approvisionnement, ktep-pci)</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://www.energiemines.gov.tn/fileadmin/docs-u1/Chiffres_cl%C3%A9s_%C3%A9nergie_2024.pdf</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Context for the learning guide; not used by the model. For the 2023-2024 change (-25%).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add the 2027-2030 pathway with Tunisia's real building pace
Each year starts from the year before: committed plants switch on in their commissioning year, and on top of them the model may add at most 268 MW of solar a year (Tunisia's fastest year so far), no wind before 2029 then 75 MW a year, and the 150 MW / 540 MWh Bazma battery from 2029. The 35% target is reported, not forced. Savings and shifting ramp up to their full value in 2030. New sourced rows and labelled assumptions in the register; Voltalia's 2026 Gabes award added to the committed projects.
</commit_message>
<xml_diff>
--- a/data/assumptions_register.xlsx
+++ b/data/assumptions_register.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3846,6 +3846,391 @@
       <c r="I75" t="inlineStr">
         <is>
           <t>Context for the learning guide; not used by the model. For the 2023-2024 change (-25%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>solar_capacity_2024_mw</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Installed solar capacity at end-2024 (all sizes)</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>773</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Enerdata, 'France's Voltalia expands Tunisian portfolio with 132 MW solar project' (4 Feb 2026)</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://www.enerdata.net/publications/daily-energy-news/frances-voltalia-expands-tunisian-portfolio-132-mw-solar-project.html</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>'solar capacity reached 773 MW at year-end, representing a 53% increase compared to 2023'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>solar_growth_2024</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Growth of installed solar capacity in 2024</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Enerdata, 'France's Voltalia expands Tunisian portfolio with 132 MW solar project' (4 Feb 2026)</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://www.enerdata.net/publications/daily-energy-news/frances-voltalia-expands-tunisian-portfolio-132-mw-solar-project.html</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Same sentence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>pathway_solar_extra_mw_per_year</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Pathway: most new solar per year beyond the committed projects</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>268</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>MW/yr</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>assumption</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Tunisia's fastest year so far: 773 - 773/1.53 = 268 MW added in 2024 (solar_capacity_2024_mw, solar_growth_2024). Covers rooftops, small plants and any new tender.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>pathway_wind_first_year</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Pathway: first year new wind (beyond committed) can come online</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>2029</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>assumption</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>2 GW of wind tenders cleared Jan 2026 with measurements pending (Industrial Info, Jan 2026); award to operation takes about two years (Voltalia Gabes: awarded 2026, operation 2028, Enerdata 4 Feb 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>pathway_wind_extra_mw_per_year</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Pathway: most new wind per year from the first wind year</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>75</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>MW/yr</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>assumption</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Enerdata, 'Tunisia launches a tender for 1.7 GW of renewables' (5 Jan 2023)</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://www.enerdata.net/publications/daily-energy-news/tunisia-launches-tender-17-gw-renewables.html</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>The 1.7 GW tender's wind lots were 75 MW each ('eight 75 MW wind projects'); one lot per year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>pathway_battery_first_year</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Pathway: first year a large battery can come online</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>2029</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>assumption</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Mercom, 'Tunisia invites bids for 300 MW solar plus 150 MW/540 MWh battery storage project' (Mar 2026)</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://www.mercomindia.com/tunisia-invites-bids-for-300-mw-solar-plus-150-mw-540-mwh-battery-storage-project</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Bazma solar-plus-storage tender, bids due 14 Oct 2026; about two years from award to operation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>pathway_battery_mw</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Pathway: most battery power available from the first battery year</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>150</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>assumption</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Mercom, 'Tunisia invites bids for 300 MW solar plus 150 MW/540 MWh battery storage project' (Mar 2026)</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://www.mercomindia.com/tunisia-invites-bids-for-300-mw-solar-plus-150-mw-540-mwh-battery-storage-project</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Size of the Bazma battery (150 MW / 540 MWh).</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>anme_demand_cut_2030</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ANME goal: cut in energy demand by 2030</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>sourced</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>AllAfrica / La Presse, ANME announcement of the national energy-conservation strategy (24 Oct 2025)</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://fr.allafrica.com/stories/202510240478.html</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Context: the national energy-conservation strategy; not used directly by the model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>pathway_battery_mwh</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Pathway: most battery energy available from the first battery year</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>540</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>assumption</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Mercom, 'Tunisia invites bids for 300 MW solar plus 150 MW/540 MWh battery storage project' (Mar 2026)</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://www.mercomindia.com/tunisia-invites-bids-for-300-mw-solar-plus-150-mw-540-mwh-battery-storage-project</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Energy of the Bazma battery (150 MW / 540 MWh).</t>
         </is>
       </c>
     </row>

</xml_diff>